<commit_message>
Initial Glider Design v7.0
- Python
</commit_message>
<xml_diff>
--- a/02_Glider_Design/C_results/nausicaa_results.xlsx
+++ b/02_Glider_Design/C_results/nausicaa_results.xlsx
@@ -457,7 +457,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>645d7d7-dirty</t>
+          <t>932d1eb-dirty</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -490,7 +490,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.60949299021477</v>
+        <v>0.4861186254890529</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -505,7 +505,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>6.5</v>
+        <v>4</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -520,7 +520,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>3.033630367943769</v>
+        <v>4.948056657833936</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -535,7 +535,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>-3.148148880762615e-16</v>
+        <v>2.474325229812098e-16</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -550,7 +550,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0.345341840795361</v>
+        <v>0.8836120799594211</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -565,7 +565,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>-1.532946721359457e-14</v>
+        <v>-7.944965084580525e-15</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
@@ -580,7 +580,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>0.09078789191347983</v>
+        <v>0.07007773737851213</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
@@ -595,7 +595,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>90.78789191347983</v>
+        <v>70.07773737851213</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
@@ -610,7 +610,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.2001530403024191</v>
+        <v>0.1544949651126453</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -625,7 +625,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.02500000998616425</v>
+        <v>-9.998916929839549e-09</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
@@ -640,7 +640,7 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>0.5813115556402076</v>
+        <v>0.4719469279513472</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
@@ -655,7 +655,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>11.18161141661032</v>
+        <v>8.475529143122294</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
@@ -670,7 +670,7 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>8.172007954129075</v>
+        <v>4.687449301023788</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
@@ -685,7 +685,7 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>41821.22376080244</v>
+        <v>39550.96498477143</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
@@ -700,7 +700,7 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>0.04999999010101803</v>
+        <v>0.1000000098892254</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
@@ -715,7 +715,7 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>0.6721799329461787</v>
+        <v>0.4999999900567649</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
@@ -730,7 +730,7 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>0.02999999002751742</v>
+        <v>0.05000000993196219</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
@@ -745,7 +745,7 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>1.295592516496379</v>
+        <v>0.9369224915798031</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
@@ -760,7 +760,7 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>243.3298652796471</v>
+        <v>86.48660579717323</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
@@ -775,7 +775,7 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>0.005324428692743563</v>
+        <v>0.01083315136423617</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
@@ -790,7 +790,7 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>0.01360115845257378</v>
+        <v>0.01065190338180691</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
@@ -836,7 +836,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>1.15962593950728</v>
+        <v>1.01542662201922</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -851,7 +851,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.09398320197010014</v>
+        <v>0.1444321744683164</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -866,7 +866,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.1089853588824799</v>
+        <v>0.1466602750312531</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -881,7 +881,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>12.33865111210197</v>
+        <v>7.03047382452842</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -896,7 +896,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.850000005846944</v>
+        <v>0.8500000084288141</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -911,7 +911,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.1799999981912146</v>
+        <v>0.2232511737645986</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -926,7 +926,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0.04499999954780364</v>
+        <v>0.05581279344114965</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -941,7 +941,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>0.008099999837209312</v>
+        <v>0.01246027164681775</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
@@ -956,7 +956,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>0.09373134698678634</v>
+        <v>0.131355066259813</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
@@ -971,7 +971,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.04686567349339317</v>
+        <v>0.06567753312990651</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
@@ -986,7 +986,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.00439278270397867</v>
+        <v>0.008627076716059934</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -1118,79 +1118,79 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>ballast</t>
+          <t>wing</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.02500000998616425</v>
+        <v>0.01935915630412541</v>
       </c>
       <c r="C2" t="n">
-        <v>25.00000998616425</v>
+        <v>19.35915630412541</v>
       </c>
       <c r="D2" t="n">
-        <v>0.02819496059103004</v>
+        <v>0.07221608723415818</v>
       </c>
       <c r="E2" t="n">
         <v>0</v>
       </c>
       <c r="F2" t="n">
-        <v>0</v>
+        <v>0.04408174561703111</v>
       </c>
       <c r="G2" t="n">
-        <v>0</v>
+        <v>0.001613288869751387</v>
       </c>
       <c r="H2" t="n">
-        <v>0</v>
+        <v>3.472586709721808e-05</v>
       </c>
       <c r="I2" t="n">
-        <v>0</v>
+        <v>0.001647963112431794</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>wing</t>
+          <t>battery</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.01438606737248734</v>
+        <v>0.013</v>
       </c>
       <c r="C3" t="n">
-        <v>14.38606737248734</v>
+        <v>13</v>
       </c>
       <c r="D3" t="n">
-        <v>0.04699160098505007</v>
+        <v>0.03610804361707909</v>
       </c>
       <c r="E3" t="n">
         <v>0</v>
       </c>
       <c r="F3" t="n">
-        <v>0.05034173279268531</v>
+        <v>0</v>
       </c>
       <c r="G3" t="n">
-        <v>0.001563525370303809</v>
+        <v>0</v>
       </c>
       <c r="H3" t="n">
-        <v>1.09375663237814e-05</v>
+        <v>0</v>
       </c>
       <c r="I3" t="n">
-        <v>0.001574424573781264</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>battery</t>
+          <t>servos</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.013</v>
+        <v>0.008800000000000001</v>
       </c>
       <c r="C4" t="n">
-        <v>13</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="D4" t="n">
-        <v>0.02349580049252504</v>
+        <v>0.04332965234049491</v>
       </c>
       <c r="E4" t="n">
         <v>0</v>
@@ -1211,17 +1211,17 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>servos</t>
+          <t>boom</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.008800000000000001</v>
+        <v>0.008640000075859326</v>
       </c>
       <c r="C5" t="n">
-        <v>8.800000000000001</v>
+        <v>8.640000075859327</v>
       </c>
       <c r="D5" t="n">
-        <v>0.02819496059103004</v>
+        <v>0.370000004214407</v>
       </c>
       <c r="E5" t="n">
         <v>0</v>
@@ -1242,17 +1242,17 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>boom</t>
+          <t>pod</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.008640000052622495</v>
+        <v>0.007</v>
       </c>
       <c r="C6" t="n">
-        <v>8.640000052622495</v>
+        <v>7</v>
       </c>
       <c r="D6" t="n">
-        <v>0.370000002923472</v>
+        <v>-0.095</v>
       </c>
       <c r="E6" t="n">
         <v>0</v>
@@ -1273,79 +1273,79 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>pod</t>
+          <t>glue</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.007</v>
+        <v>0.005190943509519417</v>
       </c>
       <c r="C7" t="n">
-        <v>7</v>
+        <v>5.190943509519417</v>
       </c>
       <c r="D7" t="n">
-        <v>-0.095</v>
+        <v>0.1008297531147197</v>
       </c>
       <c r="E7" t="n">
         <v>0</v>
       </c>
       <c r="F7" t="n">
-        <v>0</v>
+        <v>0.01401640080971708</v>
       </c>
       <c r="G7" t="n">
-        <v>0</v>
+        <v>0.0001318557759432717</v>
       </c>
       <c r="H7" t="n">
-        <v>0</v>
+        <v>0.0002106330468472504</v>
       </c>
       <c r="I7" t="n">
-        <v>0</v>
+        <v>0.0003377192267915532</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>glue</t>
+          <t>receiver</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0.006725029030628136</v>
+        <v>0.005</v>
       </c>
       <c r="C8" t="n">
-        <v>6.725029030628136</v>
+        <v>5</v>
       </c>
       <c r="D8" t="n">
-        <v>0.06507940084187656</v>
+        <v>-0.1</v>
       </c>
       <c r="E8" t="n">
         <v>0</v>
       </c>
       <c r="F8" t="n">
-        <v>0.008857665981638807</v>
+        <v>0</v>
       </c>
       <c r="G8" t="n">
-        <v>0.0001277462433729217</v>
+        <v>0</v>
       </c>
       <c r="H8" t="n">
-        <v>0.0001736723623582004</v>
+        <v>0</v>
       </c>
       <c r="I8" t="n">
-        <v>0.0002964335821785161</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>receiver</t>
+          <t>htail_surfaces</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>0.005</v>
+        <v>0.001233566893034957</v>
       </c>
       <c r="C9" t="n">
-        <v>5</v>
+        <v>1.233566893034957</v>
       </c>
       <c r="D9" t="n">
-        <v>-0.1</v>
+        <v>0.8779064051493889</v>
       </c>
       <c r="E9" t="n">
         <v>0</v>
@@ -1354,13 +1354,13 @@
         <v>0</v>
       </c>
       <c r="G9" t="n">
-        <v>0</v>
+        <v>5.124451369081958e-06</v>
       </c>
       <c r="H9" t="n">
-        <v>0</v>
+        <v>3.211455622892876e-07</v>
       </c>
       <c r="I9" t="n">
-        <v>0</v>
+        <v>5.443746581031693e-06</v>
       </c>
     </row>
     <row r="10">
@@ -1376,7 +1376,7 @@
         <v>1</v>
       </c>
       <c r="D10" t="n">
-        <v>0.425000002923472</v>
+        <v>0.425000004214407</v>
       </c>
       <c r="E10" t="n">
         <v>0</v>
@@ -1397,63 +1397,63 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>htail_surfaces</t>
+          <t>vtail_surfaces</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.000801899983883722</v>
+        <v>0.0008540805948899335</v>
       </c>
       <c r="C11" t="n">
-        <v>0.801899983883722</v>
+        <v>0.8540805948899336</v>
       </c>
       <c r="D11" t="n">
-        <v>0.8725000056208458</v>
+        <v>0.8828387749937673</v>
       </c>
       <c r="E11" t="n">
         <v>0</v>
       </c>
       <c r="F11" t="n">
-        <v>0</v>
+        <v>0.06567753312990651</v>
       </c>
       <c r="G11" t="n">
-        <v>2.165731337960013e-06</v>
+        <v>1.228677029415095e-06</v>
       </c>
       <c r="H11" t="n">
-        <v>1.35922044548669e-07</v>
+        <v>1.535045586211159e-06</v>
       </c>
       <c r="I11" t="n">
-        <v>2.300450532532856e-06</v>
+        <v>3.076496776883993e-07</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>vtail_surfaces</t>
+          <t>ballast</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.0004348854876938883</v>
+        <v>-9.998916929839549e-09</v>
       </c>
       <c r="C12" t="n">
-        <v>0.4348854876938884</v>
+        <v>-9.998916929839549e-06</v>
       </c>
       <c r="D12" t="n">
-        <v>0.8734328425936406</v>
+        <v>0.04332965234049491</v>
       </c>
       <c r="E12" t="n">
         <v>0</v>
       </c>
       <c r="F12" t="n">
-        <v>0.04686567349339317</v>
+        <v>0</v>
       </c>
       <c r="G12" t="n">
-        <v>3.18719072207944e-07</v>
+        <v>0</v>
       </c>
       <c r="H12" t="n">
-        <v>3.97991135115217e-07</v>
+        <v>0</v>
       </c>
       <c r="I12" t="n">
-        <v>7.992439113881381e-08</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -1489,7 +1489,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.02824176748593176</v>
+        <v>0.05643440872268236</v>
       </c>
     </row>
     <row r="3">
@@ -1499,7 +1499,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.5582584650035635</v>
+        <v>1.438220849459783</v>
       </c>
     </row>
     <row r="4">
@@ -1509,7 +1509,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>9.462885680624051e-07</v>
+        <v>8.9435818077161e-06</v>
       </c>
     </row>
     <row r="5">
@@ -1519,7 +1519,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>-0.001820858179731738</v>
+        <v>0.004000000909568091</v>
       </c>
     </row>
     <row r="6">
@@ -1529,7 +1529,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>-0.151993529865866</v>
+        <v>-0.2779008321205922</v>
       </c>
     </row>
     <row r="7">
@@ -1539,7 +1539,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>-0.0001342529718818819</v>
+        <v>-0.0001888888080808782</v>
       </c>
     </row>
     <row r="8">
@@ -1549,7 +1549,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0.3157884697459488</v>
+        <v>0.4783114758039694</v>
       </c>
     </row>
     <row r="9">
@@ -1559,7 +1559,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>7.053095717966677</v>
+        <v>5.798504610333541</v>
       </c>
     </row>
     <row r="10">
@@ -1569,7 +1569,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>-2.362218317472915e-05</v>
+        <v>6.878875040077161e-06</v>
       </c>
     </row>
     <row r="11">
@@ -1579,7 +1579,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>-0.01336292844966724</v>
+        <v>0.006383865311654358</v>
       </c>
     </row>
     <row r="12">
@@ -1589,7 +1589,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.8972402557599345</v>
+        <v>-0.06750078826839312</v>
       </c>
     </row>
     <row r="13">
@@ -1599,7 +1599,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>-0.0001163375792367916</v>
+        <v>6.370983379744288e-05</v>
       </c>
     </row>
     <row r="14">
@@ -1609,7 +1609,7 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>5.229757316291048e-17</v>
+        <v>1.36280273604308e-17</v>
       </c>
     </row>
     <row r="15">
@@ -1619,7 +1619,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>-9.638135169921558e-22</v>
+        <v>-1.54614635436273e-22</v>
       </c>
     </row>
     <row r="16">
@@ -1629,7 +1629,7 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>-0.2872467427726584</v>
+        <v>-0.262859136343078</v>
       </c>
     </row>
     <row r="17">
@@ -1639,7 +1639,7 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>-0.6057466955043023</v>
+        <v>-0.4898064667341854</v>
       </c>
     </row>
     <row r="18">
@@ -1649,7 +1649,7 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>2.396241335171523e-17</v>
+        <v>6.886551128437982e-18</v>
       </c>
     </row>
     <row r="19">
@@ -1659,7 +1659,7 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>0.1343180177490436</v>
+        <v>0.2193366675598729</v>
       </c>
     </row>
     <row r="20">
@@ -1669,7 +1669,7 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>1.725545558849204e-18</v>
+        <v>6.498174511321335e-19</v>
       </c>
     </row>
     <row r="21">
@@ -1679,7 +1679,7 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>2.15745950767817e-19</v>
+        <v>-5.027597466942898e-19</v>
       </c>
     </row>
     <row r="22">
@@ -1689,7 +1689,7 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>-0.3018667952492765</v>
+        <v>-0.2439029982715797</v>
       </c>
     </row>
     <row r="23">
@@ -1699,7 +1699,7 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>-1.144754916878425</v>
+        <v>-0.9145964757529272</v>
       </c>
     </row>
     <row r="24">
@@ -1709,7 +1709,7 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>3.075196367056272e-18</v>
+        <v>-5.500116102087741e-18</v>
       </c>
     </row>
     <row r="25">
@@ -1719,7 +1719,7 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>0.02306446452892491</v>
+        <v>0.04821558204849526</v>
       </c>
     </row>
     <row r="26">
@@ -1729,7 +1729,7 @@
         </is>
       </c>
       <c r="B26" t="n">
-        <v>1.943361263156383e-14</v>
+        <v>1.26481120295569e-13</v>
       </c>
     </row>
     <row r="27">
@@ -1739,7 +1739,7 @@
         </is>
       </c>
       <c r="B27" t="n">
-        <v>-0.3526547160798665</v>
+        <v>-0.5798505183760735</v>
       </c>
     </row>
     <row r="28">
@@ -1749,7 +1749,7 @@
         </is>
       </c>
       <c r="B28" t="n">
-        <v>-6.503432824197187e-06</v>
+        <v>2.581053145020834e-06</v>
       </c>
     </row>
     <row r="29">
@@ -1759,7 +1759,7 @@
         </is>
       </c>
       <c r="B29" t="n">
-        <v>-0.004120815588269226</v>
+        <v>0.002163318530967793</v>
       </c>
     </row>
     <row r="30">
@@ -1769,7 +1769,7 @@
         </is>
       </c>
       <c r="B30" t="n">
-        <v>-63.14464862925413</v>
+        <v>-29.33297990530776</v>
       </c>
     </row>
     <row r="31">
@@ -1779,7 +1779,7 @@
         </is>
       </c>
       <c r="B31" t="n">
-        <v>-0.0001371512796438799</v>
+        <v>-0.0001530424517202103</v>
       </c>
     </row>
     <row r="32">
@@ -1789,7 +1789,7 @@
         </is>
       </c>
       <c r="B32" t="n">
-        <v>-3.600976924317262e-17</v>
+        <v>-9.716636602208142e-18</v>
       </c>
     </row>
     <row r="33">
@@ -1799,7 +1799,7 @@
         </is>
       </c>
       <c r="B33" t="n">
-        <v>1.210096493883213e-20</v>
+        <v>-4.342007604553401e-20</v>
       </c>
     </row>
     <row r="34">
@@ -1809,7 +1809,7 @@
         </is>
       </c>
       <c r="B34" t="n">
-        <v>0.04598430542773188</v>
+        <v>0.09957879373496006</v>
       </c>
     </row>
     <row r="35">
@@ -1819,7 +1819,7 @@
         </is>
       </c>
       <c r="B35" t="n">
-        <v>-0.06093555807088765</v>
+        <v>0.005594368626645732</v>
       </c>
     </row>
     <row r="36">
@@ -1829,7 +1829,7 @@
         </is>
       </c>
       <c r="B36" t="n">
-        <v>-1.627519054399944e-17</v>
+        <v>-5.398133074725084e-18</v>
       </c>
     </row>
     <row r="37">
@@ -1839,7 +1839,7 @@
         </is>
       </c>
       <c r="B37" t="n">
-        <v>-0.09264074246226461</v>
+        <v>-0.1488566314128205</v>
       </c>
     </row>
     <row r="38">
@@ -1849,7 +1849,7 @@
         </is>
       </c>
       <c r="B38" t="n">
-        <v>0.07965123956703249</v>
+        <v>0.08111146597243066</v>
       </c>
     </row>
     <row r="39">
@@ -1859,7 +1859,7 @@
         </is>
       </c>
       <c r="B39" t="n">
-        <v>0.009800965861908175</v>
+        <v>0.0193538902475611</v>
       </c>
     </row>
     <row r="40">
@@ -1869,7 +1869,7 @@
         </is>
       </c>
       <c r="B40" t="n">
-        <v>0.06985027370512431</v>
+        <v>0.06175757572486956</v>
       </c>
     </row>
     <row r="41">
@@ -1879,7 +1879,7 @@
         </is>
       </c>
       <c r="B41" t="n">
-        <v>-0.03240564863495038</v>
+        <v>-0.0215137694811276</v>
       </c>
     </row>
     <row r="42">
@@ -1889,7 +1889,7 @@
         </is>
       </c>
       <c r="B42" t="n">
-        <v>0.03240564863495038</v>
+        <v>0.0215137694811276</v>
       </c>
     </row>
     <row r="43">
@@ -1899,7 +1899,7 @@
         </is>
       </c>
       <c r="B43" t="n">
-        <v>-0.07965123956703249</v>
+        <v>-0.08111146597243066</v>
       </c>
     </row>
     <row r="44">
@@ -1909,7 +1909,7 @@
         </is>
       </c>
       <c r="B44" t="n">
-        <v>0.8906292096898943</v>
+        <v>0.6874625936907084</v>
       </c>
     </row>
     <row r="45">
@@ -1919,7 +1919,7 @@
         </is>
       </c>
       <c r="B45" t="n">
-        <v>5.643454363768099e-18</v>
+        <v>9.483708294407718e-19</v>
       </c>
     </row>
     <row r="46">
@@ -1929,7 +1929,7 @@
         </is>
       </c>
       <c r="B46" t="n">
-        <v>-5.643454363768099e-18</v>
+        <v>-9.483708294407718e-19</v>
       </c>
     </row>
     <row r="47">
@@ -1939,7 +1939,7 @@
         </is>
       </c>
       <c r="B47" t="n">
-        <v>-5.971512479971581e-19</v>
+        <v>-2.782997315972464e-19</v>
       </c>
     </row>
     <row r="48">
@@ -1949,7 +1949,7 @@
         </is>
       </c>
       <c r="B48" t="n">
-        <v>1.474966653857061e-16</v>
+        <v>1.958715086302754e-17</v>
       </c>
     </row>
     <row r="49">
@@ -1961,11 +1961,11 @@
       <c r="B49" t="inlineStr">
         <is>
           <t>[AeroComponentResults(
-	L=0.00039918417148410775,
+	L=0.0003914046783731243,
 	Y=0.0,
-	D=0.001915024915027601,
+	D=0.0008358760882080647,
 	l_b=-0.0,
-	m_b=-0.00016370490668699133,
+	m_b=-0.0001383265370471261,
 	n_b=-0.0,
 	span_effective=0.004055451774444796, oswalds_efficiency=0.95,
 )]</t>
@@ -1979,7 +1979,7 @@
         </is>
       </c>
       <c r="B50" t="n">
-        <v>5.643454363768099e-18</v>
+        <v>9.483708294407718e-19</v>
       </c>
     </row>
     <row r="51">
@@ -1989,7 +1989,7 @@
         </is>
       </c>
       <c r="B51" t="n">
-        <v>5.15115294169588e-15</v>
+        <v>2.625596138075559e-14</v>
       </c>
     </row>
     <row r="52">
@@ -1999,7 +1999,7 @@
         </is>
       </c>
       <c r="B52" t="n">
-        <v>-1.177711526256052e-16</v>
+        <v>-1.418086679229076e-17</v>
       </c>
     </row>
     <row r="53">
@@ -2011,29 +2011,29 @@
       <c r="B53" t="inlineStr">
         <is>
           <t>[AeroComponentResults(
-	L=0.844362156645189,
+	L=0.6315308867064954,
 	Y=0.0,
-	D=0.061000032511265775,
+	D=0.05421727206110085,
 	l_b=-0.0,
-	m_b=0.03675919853049462,
+	m_b=0.04270644773075434,
 	n_b=-0.0,
-	span_effective=1.1421424391871897, oswalds_efficiency=0.7631362337472126,
+	span_effective=1.0001171924296708, oswalds_efficiency=0.7929621089044373,
 ), AeroComponentResults(
-	L=0.045867868873221466,
+	L=0.0555403023058398,
 	Y=0.0,
-	D=0.00486823060563684,
+	D=0.005030575822673577,
 	l_b=-0.0,
-	m_b=-0.036587125278178444,
+	m_b=-0.0425443386386366,
 	n_b=-0.0,
-	span_effective=0.17999999819121457, oswalds_efficiency=0.8106853777008906,
+	span_effective=0.2232511737645986, oswalds_efficiency=0.8106853777008906,
 ), AeroComponentResults(
-	L=-0.0,
-	Y=1.474966653857061e-16,
-	D=0.0020669856731941006,
-	l_b=5.643454363768099e-18,
-	m_b=-8.368345624034154e-06,
-	n_b=-1.177711526256052e-16,
-	span_effective=0.09373134698678634, oswalds_efficiency=0.8232692748986458,
+	L=2.710505431213761e-20,
+	Y=1.958715086302754e-17,
+	D=0.0016738517528870596,
+	l_b=9.483708294407718e-19,
+	m_b=-2.3782555044355553e-05,
+	n_b=-1.4180866792290764e-17,
+	span_effective=0.13135506625981302, oswalds_efficiency=0.8232692748986458,
 )]</t>
         </is>
       </c>
@@ -2045,7 +2045,7 @@
         </is>
       </c>
       <c r="B54" t="n">
-        <v>0.06977856001004355</v>
+        <v>0.1152729719898737</v>
       </c>
     </row>
     <row r="55">
@@ -2055,7 +2055,7 @@
         </is>
       </c>
       <c r="B55" t="n">
-        <v>0.2507197770198829</v>
+        <v>0.4855033069951758</v>
       </c>
     </row>
   </sheetData>
@@ -2111,10 +2111,10 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.8906292096898943</v>
+        <v>0.6874625936907084</v>
       </c>
       <c r="C2" t="n">
-        <v>0.8906292196712372</v>
+        <v>0.687462603683204</v>
       </c>
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="n">
@@ -2131,7 +2131,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.07965123956703249</v>
+        <v>0.08111146597243066</v>
       </c>
       <c r="C3" t="n">
         <v>0.001</v>
@@ -2151,7 +2151,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>1.943361263156383e-14</v>
+        <v>1.26481120295569e-13</v>
       </c>
       <c r="C4" t="n">
         <v>0</v>
@@ -2173,7 +2173,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>1.725545558849204e-18</v>
+        <v>6.498174511321335e-19</v>
       </c>
       <c r="C5" t="n">
         <v>0</v>
@@ -2195,7 +2195,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>-3.600976924317262e-17</v>
+        <v>-9.716636602208142e-18</v>
       </c>
       <c r="C6" t="n">
         <v>0</v>
@@ -2217,7 +2217,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.3157884697459488</v>
+        <v>0.4783114758039694</v>
       </c>
       <c r="C7" t="inlineStr"/>
       <c r="D7" t="n">
@@ -2237,7 +2237,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>3.033630367943769</v>
+        <v>4.948056657833936</v>
       </c>
       <c r="C8" t="inlineStr"/>
       <c r="D8" t="n">
@@ -2257,7 +2257,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>11.18161141661032</v>
+        <v>8.475529143122294</v>
       </c>
       <c r="C9" t="n">
         <v>8</v>
@@ -2277,7 +2277,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>8.172007954129075</v>
+        <v>4.687449301023788</v>
       </c>
       <c r="C10" t="n">
         <v>2</v>
@@ -2297,7 +2297,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>8.172007954129075</v>
+        <v>4.687449301023788</v>
       </c>
       <c r="C11" t="inlineStr"/>
       <c r="D11" t="n">
@@ -2317,7 +2317,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>41821.22376080244</v>
+        <v>39550.96498477143</v>
       </c>
       <c r="C12" t="n">
         <v>20000</v>
@@ -2337,7 +2337,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.04999999010101803</v>
+        <v>0.1000000098892254</v>
       </c>
       <c r="C13" t="n">
         <v>0.05</v>
@@ -2357,7 +2357,7 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>0.04999999010101803</v>
+        <v>0.1000000098892254</v>
       </c>
       <c r="C14" t="inlineStr"/>
       <c r="D14" t="n">
@@ -2377,7 +2377,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>0.6721799329461787</v>
+        <v>0.4999999900567649</v>
       </c>
       <c r="C15" t="n">
         <v>0.5</v>
@@ -2397,7 +2397,7 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>0.6721799329461787</v>
+        <v>0.4999999900567649</v>
       </c>
       <c r="C16" t="inlineStr"/>
       <c r="D16" t="n">
@@ -2417,7 +2417,7 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>0.02999999002751742</v>
+        <v>0.05000000993196219</v>
       </c>
       <c r="C17" t="n">
         <v>0.03</v>
@@ -2437,7 +2437,7 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>0.02999999002751742</v>
+        <v>0.05000000993196219</v>
       </c>
       <c r="C18" t="inlineStr"/>
       <c r="D18" t="n">
@@ -2457,7 +2457,7 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>-0.3018667952492765</v>
+        <v>-0.2439029982715797</v>
       </c>
       <c r="C19" t="inlineStr"/>
       <c r="D19" t="n">
@@ -2477,7 +2477,7 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>0.04598430542773188</v>
+        <v>0.09957879373496006</v>
       </c>
       <c r="C20" t="n">
         <v>0</v>
@@ -2497,7 +2497,7 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>-63.14464862925413</v>
+        <v>-29.33297990530776</v>
       </c>
       <c r="C21" t="inlineStr"/>
       <c r="D21" t="n">
@@ -2517,7 +2517,7 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>1.295592516496379</v>
+        <v>0.9369224915798031</v>
       </c>
       <c r="C22" t="n">
         <v>0.6</v>
@@ -2537,7 +2537,7 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>243.3298652796471</v>
+        <v>86.48660579717323</v>
       </c>
       <c r="C23" t="n">
         <v>2</v>
@@ -2557,7 +2557,7 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>0.005324428692743563</v>
+        <v>0.01083315136423617</v>
       </c>
       <c r="C24" t="inlineStr"/>
       <c r="D24" t="n">
@@ -2577,7 +2577,7 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>0.001088092676205903</v>
+        <v>0.0008521522705445529</v>
       </c>
       <c r="C25" t="inlineStr"/>
       <c r="D25" t="n">
@@ -2597,7 +2597,7 @@
         </is>
       </c>
       <c r="B26" t="n">
-        <v>5.116811316151226e-06</v>
+        <v>9.45951493738948e-06</v>
       </c>
       <c r="C26" t="inlineStr"/>
       <c r="D26" t="n">
@@ -2617,7 +2617,7 @@
         </is>
       </c>
       <c r="B27" t="n">
-        <v>1.746095152991352e-19</v>
+        <v>9.432178633127867e-20</v>
       </c>
       <c r="C27" t="inlineStr"/>
       <c r="D27" t="n">

</xml_diff>

<commit_message>
Initial Glider Design v7.1
- Python
- Add Flight Arena constriant
</commit_message>
<xml_diff>
--- a/02_Glider_Design/C_results/nausicaa_results.xlsx
+++ b/02_Glider_Design/C_results/nausicaa_results.xlsx
@@ -12,6 +12,7 @@
     <sheet name="MassBreakdown" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Aerodynamics" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="Constraints" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="DesignPoints" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -429,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C24"/>
+  <dimension ref="A1:C31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -457,7 +458,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>a99069b-dirty</t>
+          <t>5cb9697-dirty</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -490,7 +491,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.486118625467693</v>
+        <v>0.3829646626678594</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -501,7 +502,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>design_speed_mps</t>
+          <t>v_nom_mps</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -516,26 +517,26 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>alpha_trim_deg</t>
+          <t>v_turn_mps</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>4.948056657649936</v>
+        <v>3</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>deg</t>
+          <t>m/s</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>delta_a_trim_deg</t>
+          <t>turn_bank_deg</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>6.014083662992938e-17</v>
+        <v>50</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -546,176 +547,176 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>delta_e_trim_deg</t>
+          <t>arena_width_m</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0.883612080032152</v>
+        <v>4.8</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>deg</t>
+          <t>m</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>delta_r_trim_deg</t>
+          <t>wall_clearance_m</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>-8.295475058712677e-15</v>
+        <v>0.5</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>deg</t>
+          <t>m</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>mass_total_kg</t>
+          <t>alpha_trim_deg</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>0.07007773737740047</v>
+        <v>3.265624972678735</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>kg</t>
+          <t>deg</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>mass_total_g</t>
+          <t>delta_a_trim_deg</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>70.07773737740047</v>
+        <v>1.732786463659694e-16</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>g</t>
+          <t>deg</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>mass_total_lbm</t>
+          <t>delta_e_trim_deg</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.1544949651101946</v>
+        <v>0.7295201394751571</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>lbm</t>
+          <t>deg</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>ballast_mass_kg</t>
+          <t>delta_r_trim_deg</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>-1.000074676233832e-08</v>
+        <v>1.035118855641136e-15</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>kg</t>
+          <t>deg</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>sink_rate_mps</t>
+          <t>mass_total_kg</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>0.4719469279309158</v>
+        <v>0.08907177338753518</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>m/s</t>
+          <t>kg</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>L_over_D</t>
+          <t>mass_total_g</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>8.475529143488501</v>
+        <v>89.07177338753517</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>g</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>wing_loading_n_m2</t>
+          <t>mass_total_lbm</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>4.687449300794357</v>
+        <v>0.1963696465783478</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>N/m^2</t>
+          <t>lbm</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>reynolds_wing</t>
+          <t>ballast_mass_kg</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>39550.96498607255</v>
+        <v>0.001248044074387546</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>kg</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>static_margin</t>
+          <t>sink_rate_mps</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>0.1000000099170008</v>
+        <v>0.3645446504338175</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>MAC fraction</t>
+          <t>m/s</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>tail_volume_horizontal</t>
+          <t>L_over_D</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>0.4999999900541847</v>
+        <v>10.97259265635919</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
@@ -726,73 +727,178 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>tail_volume_vertical</t>
+          <t>turn_radius_m</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>0.0500000099349265</v>
+        <v>0.769816175392</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>m</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>roll_rate_ss_radps</t>
+          <t>turn_footprint_lhs_m</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>0.9369224915803962</v>
+        <v>2.080046038462513</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>rad/s</t>
+          <t>m</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>roll_accel0_rad_s2</t>
+          <t>turn_CL</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>86.48660579196596</v>
+        <v>0.3528117324472714</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>rad/s^2</t>
+          <t>-</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>roll_tau_s</t>
+          <t>wing_loading_n_m2</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>0.01083315136489528</v>
+        <v>3.467824177017998</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>s</t>
+          <t>N/m^2</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
+          <t>reynolds_wing</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>41933.23691995171</v>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>static_margin</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>0.04999999020698476</v>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>MAC fraction</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>tail_volume_horizontal</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>0.7000000080815174</v>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>tail_volume_vertical</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>0.02999999000825085</v>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>roll_rate_ss_radps</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>0.5999999902481539</v>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>rad/s</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>roll_accel0_rad_s2</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>64.60823526290454</v>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>rad/s^2</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>roll_tau_s</t>
+        </is>
+      </c>
+      <c r="B30" t="n">
+        <v>0.009286741663916792</v>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>s</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
           <t>max_servo_utilization</t>
         </is>
       </c>
-      <c r="B24" t="n">
-        <v>2.958862050697145e-05</v>
-      </c>
-      <c r="C24" t="inlineStr">
+      <c r="B31" t="n">
+        <v>5.389712043725522e-05</v>
+      </c>
+      <c r="C31" t="inlineStr">
         <is>
           <t>fraction</t>
         </is>
@@ -836,7 +942,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>1.015426622019409</v>
+        <v>1.645457929412684</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -851,7 +957,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.1444321744730677</v>
+        <v>0.1531317527442298</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -866,7 +972,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.146660275036105</v>
+        <v>0.2519718567978555</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -881,7 +987,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>7.030473824298449</v>
+        <v>10.74537383609153</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -896,7 +1002,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.8500000084297308</v>
+        <v>0.8367187539795161</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -911,7 +1017,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.2232511737712672</v>
+        <v>0.3593336687022275</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -926,7 +1032,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0.0558127934428168</v>
+        <v>0.08983341717555687</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -941,7 +1047,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>0.01246027164756214</v>
+        <v>0.03228017136575054</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
@@ -956,7 +1062,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>0.131355066265821</v>
+        <v>0.1711121863070972</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
@@ -971,7 +1077,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.06567753313291048</v>
+        <v>0.08555609315354862</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
@@ -986,7 +1092,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.008627076716849109</v>
+        <v>0.01463969015139738</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -1122,28 +1228,28 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.01935915630476586</v>
+        <v>0.03326028509731693</v>
       </c>
       <c r="C2" t="n">
-        <v>19.35915630476586</v>
+        <v>33.26028509731692</v>
       </c>
       <c r="D2" t="n">
-        <v>0.07221608723653386</v>
+        <v>0.0765658763721149</v>
       </c>
       <c r="E2" t="n">
         <v>0</v>
       </c>
       <c r="F2" t="n">
-        <v>0.04408174561703931</v>
+        <v>0.07143269271752828</v>
       </c>
       <c r="G2" t="n">
-        <v>0.001613288869805359</v>
+        <v>0.00727819775170123</v>
       </c>
       <c r="H2" t="n">
-        <v>3.472586710064994e-05</v>
+        <v>6.705939157817239e-05</v>
       </c>
       <c r="I2" t="n">
-        <v>0.001647963112489196</v>
+        <v>0.00734516844918581</v>
       </c>
     </row>
     <row r="3">
@@ -1159,7 +1265,7 @@
         <v>13</v>
       </c>
       <c r="D3" t="n">
-        <v>0.03610804361826693</v>
+        <v>0.03828293818605745</v>
       </c>
       <c r="E3" t="n">
         <v>0</v>
@@ -1190,7 +1296,7 @@
         <v>8.800000000000001</v>
       </c>
       <c r="D4" t="n">
-        <v>0.04332965234192031</v>
+        <v>0.04593952582326894</v>
       </c>
       <c r="E4" t="n">
         <v>0</v>
@@ -1215,13 +1321,13 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.008640000075867576</v>
+        <v>0.008520468785815645</v>
       </c>
       <c r="C5" t="n">
-        <v>8.640000075867576</v>
+        <v>8.520468785815645</v>
       </c>
       <c r="D5" t="n">
-        <v>0.3700000042148654</v>
+        <v>0.3633593769897581</v>
       </c>
       <c r="E5" t="n">
         <v>0</v>
@@ -1277,28 +1383,28 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.005190943509437072</v>
+        <v>0.006597909139817421</v>
       </c>
       <c r="C7" t="n">
-        <v>5.190943509437072</v>
+        <v>6.59790913981742</v>
       </c>
       <c r="D7" t="n">
-        <v>0.1008297531191905</v>
+        <v>0.1206126412622277</v>
       </c>
       <c r="E7" t="n">
         <v>0</v>
       </c>
       <c r="F7" t="n">
-        <v>0.01401640081049559</v>
+        <v>0.03031106523982323</v>
       </c>
       <c r="G7" t="n">
-        <v>0.0001318557759477139</v>
+        <v>0.0005936539099383243</v>
       </c>
       <c r="H7" t="n">
-        <v>0.0002106330468548315</v>
+        <v>0.0003385489796629639</v>
       </c>
       <c r="I7" t="n">
-        <v>0.0003377192268034254</v>
+        <v>0.0009149015983556316</v>
       </c>
     </row>
     <row r="8">
@@ -1339,13 +1445,13 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>0.001233566893108652</v>
+        <v>0.003195736965209304</v>
       </c>
       <c r="C9" t="n">
-        <v>1.233566893108652</v>
+        <v>3.195736965209304</v>
       </c>
       <c r="D9" t="n">
-        <v>0.8779064051511392</v>
+        <v>0.8816354625672945</v>
       </c>
       <c r="E9" t="n">
         <v>0</v>
@@ -1354,91 +1460,91 @@
         <v>0</v>
       </c>
       <c r="G9" t="n">
-        <v>5.124451369694181e-06</v>
+        <v>3.438870909499721e-05</v>
       </c>
       <c r="H9" t="n">
-        <v>3.211455623276033e-07</v>
+        <v>2.151541320990989e-06</v>
       </c>
       <c r="I9" t="n">
-        <v>5.443746581682121e-06</v>
+        <v>3.653545681054039e-05</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>linkages</t>
+          <t>vtail_surfaces</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>0.001</v>
+        <v>0.00144932932498834</v>
       </c>
       <c r="C10" t="n">
-        <v>1</v>
+        <v>1.44932932498834</v>
       </c>
       <c r="D10" t="n">
-        <v>0.4250000042148654</v>
+        <v>0.8794968005562904</v>
       </c>
       <c r="E10" t="n">
         <v>0</v>
       </c>
       <c r="F10" t="n">
-        <v>0</v>
+        <v>0.08555609315354862</v>
       </c>
       <c r="G10" t="n">
-        <v>0</v>
+        <v>3.537375704520944e-06</v>
       </c>
       <c r="H10" t="n">
-        <v>0</v>
+        <v>4.420360884409003e-06</v>
       </c>
       <c r="I10" t="n">
-        <v>0</v>
+        <v>8.85159173875542e-07</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>vtail_surfaces</t>
+          <t>ballast</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.0008540805949680617</v>
+        <v>0.001248044074387546</v>
       </c>
       <c r="C11" t="n">
-        <v>0.8540805949680617</v>
+        <v>1.248044074387546</v>
       </c>
       <c r="D11" t="n">
-        <v>0.882838774996186</v>
+        <v>0.04593952582326894</v>
       </c>
       <c r="E11" t="n">
         <v>0</v>
       </c>
       <c r="F11" t="n">
-        <v>0.06567753313291048</v>
+        <v>0</v>
       </c>
       <c r="G11" t="n">
-        <v>1.228677029639826e-06</v>
+        <v>0</v>
       </c>
       <c r="H11" t="n">
-        <v>1.535045586492e-06</v>
+        <v>0</v>
       </c>
       <c r="I11" t="n">
-        <v>3.076496777446261e-07</v>
+        <v>0</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>ballast</t>
+          <t>linkages</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>-1.000074676233832e-08</v>
+        <v>0.001</v>
       </c>
       <c r="C12" t="n">
-        <v>-1.000074676233832e-05</v>
+        <v>1</v>
       </c>
       <c r="D12" t="n">
-        <v>0.04332965234192031</v>
+        <v>0.4183593769897581</v>
       </c>
       <c r="E12" t="n">
         <v>0</v>
@@ -1467,7 +1573,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B55"/>
+  <dimension ref="A1:B77"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1485,487 +1591,487 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>CD</t>
+          <t>nominal_CD</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.05643440871747699</v>
+        <v>0.03224942917054652</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>CDa</t>
+          <t>nominal_CDa</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>1.438220849315466</v>
+        <v>0.6294856307726406</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>CDb</t>
+          <t>nominal_CDb</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>8.943568290358704e-06</v>
+        <v>8.340197586387651e-07</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>CDp</t>
+          <t>nominal_CDp</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.004000000916951074</v>
+        <v>-0.001820511558746352</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>CDq</t>
+          <t>nominal_CDq</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>-0.2779008320195897</v>
+        <v>-0.07529548797726575</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>CDr</t>
+          <t>nominal_CDr</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>-0.0001888888076714834</v>
+        <v>-8.380160661236591e-05</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>CL</t>
+          <t>nominal_CL</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0.4783114757805177</v>
+        <v>0.3538598496885145</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>CLa</t>
+          <t>nominal_CLa</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>5.798504609986861</v>
+        <v>7.005053025496728</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>CLb</t>
+          <t>nominal_CLb</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>6.878776442882036e-06</v>
+        <v>-2.890867534687543e-05</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>CLp</t>
+          <t>nominal_CLp</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.006383865327919124</v>
+        <v>-0.01586307811807242</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>CLq</t>
+          <t>nominal_CLq</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>-0.0675007877341538</v>
+        <v>0.3676832465103752</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>CLr</t>
+          <t>nominal_CLr</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>6.370983485215476e-05</v>
+        <v>-0.0001684725206008153</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>CY</t>
+          <t>nominal_CY</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>1.771643556959456e-17</v>
+        <v>9.422363200144823e-18</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>CYa</t>
+          <t>nominal_CYa</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>-2.009994056630966e-22</v>
+        <v>-7.075447656711423e-23</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>CYb</t>
+          <t>nominal_CYb</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>-0.2628591363433991</v>
+        <v>-0.3099907511324865</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>CYp</t>
+          <t>nominal_CYp</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>-0.4898064667066539</v>
+        <v>-0.566406099598727</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>CYq</t>
+          <t>nominal_CYq</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>8.952516464704019e-18</v>
+        <v>-2.441226992436795e-18</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>CYr</t>
+          <t>nominal_CYr</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>0.2193366675707248</v>
+        <v>0.1241092086103912</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Cl</t>
+          <t>nominal_Cl</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>9.30363791679246e-19</v>
+        <v>3.087405529260732e-19</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Cla</t>
+          <t>nominal_Cla</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>3.351590182131828e-19</v>
+        <v>-1.33346092137015e-19</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Clb</t>
+          <t>nominal_Clb</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>-0.2439029982603689</v>
+        <v>-0.2819421253289612</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Clp</t>
+          <t>nominal_Clp</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>-0.9145964756974962</v>
+        <v>-1.064729109304657</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Clq</t>
+          <t>nominal_Clq</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>3.338487439852477e-18</v>
+        <v>-1.711870338836074e-18</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Clr</t>
+          <t>nominal_Clr</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>0.04821558204955213</v>
+        <v>0.021790251455553</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Cm</t>
+          <t>nominal_Cm</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>3.039702191125778e-14</v>
+        <v>-1.491448830018954e-10</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Cma</t>
+          <t>nominal_Cma</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>-0.5798505185024612</v>
+        <v>-0.3502525826742454</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Cmb</t>
+          <t>nominal_Cmb</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>2.580938241251129e-06</v>
+        <v>-1.002744686737054e-05</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Cmp</t>
+          <t>nominal_Cmp</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>0.002163318540952959</v>
+        <v>-0.006396571209649135</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Cmq</t>
+          <t>nominal_Cmq</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>-29.3329799057312</v>
+        <v>-39.52415518558014</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Cmr</t>
+          <t>nominal_Cmr</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>-0.0001530424511486556</v>
+        <v>-0.0001389555989351931</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Cn</t>
+          <t>nominal_Cn</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>-1.362037599096439e-17</v>
+        <v>-4.05887327666648e-18</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Cna</t>
+          <t>nominal_Cna</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>2.917485264134367e-20</v>
+        <v>-7.578978318717902e-21</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Cnb</t>
+          <t>nominal_Cnb</t>
         </is>
       </c>
       <c r="B34" t="n">
-        <v>0.09957879373723921</v>
+        <v>0.03795793197254786</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Cnp</t>
+          <t>nominal_Cnp</t>
         </is>
       </c>
       <c r="B35" t="n">
-        <v>0.005594368619038168</v>
+        <v>-0.07056892499093069</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Cnq</t>
+          <t>nominal_Cnq</t>
         </is>
       </c>
       <c r="B36" t="n">
-        <v>-6.557285860509823e-18</v>
+        <v>9.725461716079436e-19</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Cnr</t>
+          <t>nominal_Cnr</t>
         </is>
       </c>
       <c r="B37" t="n">
-        <v>-0.1488566314209694</v>
+        <v>-0.05850484150544907</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>nominal_D</t>
         </is>
       </c>
       <c r="B38" t="n">
-        <v>0.08111146596763252</v>
+        <v>0.07963424090427679</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>D_induced</t>
+          <t>nominal_D_induced</t>
         </is>
       </c>
       <c r="B39" t="n">
-        <v>0.01935389024690383</v>
+        <v>0.01223295076335761</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>D_profile</t>
+          <t>nominal_D_profile</t>
         </is>
       </c>
       <c r="B40" t="n">
-        <v>0.06175757572072869</v>
+        <v>0.06740129014091917</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>F_b</t>
+          <t>nominal_F_b</t>
         </is>
       </c>
       <c r="B41" t="n">
-        <v>-0.02151376947951493</v>
+        <v>-0.02972920125926148</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>F_g</t>
+          <t>nominal_F_g</t>
         </is>
       </c>
       <c r="B42" t="n">
-        <v>0.02151376947951493</v>
+        <v>0.02972920125926148</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>F_w</t>
+          <t>nominal_F_w</t>
         </is>
       </c>
       <c r="B43" t="n">
-        <v>-0.08111146596763252</v>
+        <v>-0.07963424090427679</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>nominal_L</t>
         </is>
       </c>
       <c r="B44" t="n">
-        <v>0.6874625936797452</v>
+        <v>0.8737940869410059</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>M_b</t>
+          <t>nominal_M_b</t>
         </is>
       </c>
       <c r="B45" t="n">
-        <v>1.357811919776297e-18</v>
+        <v>1.254464203857359e-18</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>M_g</t>
+          <t>nominal_M_g</t>
         </is>
       </c>
       <c r="B46" t="n">
-        <v>-1.357811919776297e-18</v>
+        <v>-1.254464203857359e-18</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>M_w</t>
+          <t>nominal_M_w</t>
         </is>
       </c>
       <c r="B47" t="n">
-        <v>-3.61789650984088e-19</v>
+        <v>3.129665040971596e-19</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>nominal_Y</t>
         </is>
       </c>
       <c r="B48" t="n">
-        <v>2.546329612426509e-17</v>
+        <v>2.326685340691906e-17</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>fuselage_aero_components</t>
+          <t>nominal_fuselage_aero_components</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
           <t>[AeroComponentResults(
-	L=0.00039140467834894514,
+	L=0.00019699568249745332,
 	Y=0.0,
-	D=0.0008358760882064288,
+	D=0.0008275962517129193,
 	l_b=-0.0,
-	m_b=-0.00013832653703869653,
+	m_b=-8.809874262680897e-05,
 	n_b=-0.0,
 	span_effective=0.004055451774444796, oswalds_efficiency=0.95,
 )]</t>
@@ -1975,65 +2081,65 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>l_b</t>
+          <t>nominal_l_b</t>
         </is>
       </c>
       <c r="B50" t="n">
-        <v>1.357811919776297e-18</v>
+        <v>1.254464203857359e-18</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>m_b</t>
+          <t>nominal_m_b</t>
         </is>
       </c>
       <c r="B51" t="n">
-        <v>6.310056643865636e-15</v>
+        <v>-5.639640543572601e-11</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>n_b</t>
+          <t>nominal_n_b</t>
         </is>
       </c>
       <c r="B52" t="n">
-        <v>-1.987814770713083e-17</v>
+        <v>-1.649187703175008e-17</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>wing_aero_components</t>
+          <t>nominal_wing_aero_components</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
           <t>[AeroComponentResults(
-	L=0.6315308866932998,
+	L=0.783353256168381,
 	Y=0.0,
-	D=0.054217272056737584,
+	D=0.05625018019951093,
 	l_b=-0.0,
-	m_b=0.04270644773225918,
+	m_b=0.06668583167694779,
 	n_b=-0.0,
-	span_effective=1.0001171924298569, oswalds_efficiency=0.79296210890578,
+	span_effective=1.6206496155802028, oswalds_efficiency=0.7718502781381492,
 ), AeroComponentResults(
-	L=0.05554030230809642,
+	L=0.09024383509012739,
 	Y=0.0,
-	D=0.005030575822788429,
+	D=0.007883984678618852,
 	l_b=-0.0,
-	m_b=-0.04254433864017651,
+	m_b=-0.06663054752102311,
 	n_b=-0.0,
-	span_effective=0.22325117377126721, oswalds_efficiency=0.8106853777008906,
+	span_effective=0.3593336687022275, oswalds_efficiency=0.8106853777008906,
 ), AeroComponentResults(
 	L=-0.0,
-	Y=2.546329612426509e-17,
-	D=0.001673851752996247,
-	l_b=1.357811919776297e-18,
-	m_b=-2.3782555037661848e-05,
-	n_b=-1.9878147707130825e-17,
-	span_effective=0.13135506626582097, oswalds_efficiency=0.8232692748986458,
+	Y=2.326685340691906e-17,
+	D=0.0024395290110764732,
+	l_b=1.2544642038573592e-18,
+	m_b=3.2814530305724925e-05,
+	n_b=-1.6491877031750078e-17,
+	span_effective=0.17111218630709724, oswalds_efficiency=0.8232692748986458,
 )]</t>
         </is>
       </c>
@@ -2041,21 +2147,277 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>x_np</t>
+          <t>nominal_x_np</t>
         </is>
       </c>
       <c r="B54" t="n">
-        <v>0.1152729719988313</v>
+        <v>0.1282692273998176</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>x_np_lateral</t>
+          <t>nominal_x_np_lateral</t>
         </is>
       </c>
       <c r="B55" t="n">
-        <v>0.4855033070080527</v>
+        <v>0.3220966530276053</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>turn_CD</t>
+        </is>
+      </c>
+      <c r="B56" t="n">
+        <v>0.03434113097875773</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>turn_CL</t>
+        </is>
+      </c>
+      <c r="B57" t="n">
+        <v>0.3528117324472714</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>turn_CY</t>
+        </is>
+      </c>
+      <c r="B58" t="n">
+        <v>1.884426405928886e-17</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>turn_Cl</t>
+        </is>
+      </c>
+      <c r="B59" t="n">
+        <v>6.402903091352355e-19</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>turn_Cm</t>
+        </is>
+      </c>
+      <c r="B60" t="n">
+        <v>0.01094067023361572</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>turn_Cn</t>
+        </is>
+      </c>
+      <c r="B61" t="n">
+        <v>-8.517569654817715e-18</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>turn_D</t>
+        </is>
+      </c>
+      <c r="B62" t="n">
+        <v>0.04769962156816282</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>turn_D_induced</t>
+        </is>
+      </c>
+      <c r="B63" t="n">
+        <v>0.006840332530788545</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>turn_D_profile</t>
+        </is>
+      </c>
+      <c r="B64" t="n">
+        <v>0.04085928903737427</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>turn_F_b</t>
+        </is>
+      </c>
+      <c r="B65" t="n">
+        <v>-0.01970625031065464</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>turn_F_g</t>
+        </is>
+      </c>
+      <c r="B66" t="n">
+        <v>0.01970625031065464</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>turn_F_w</t>
+        </is>
+      </c>
+      <c r="B67" t="n">
+        <v>-0.04769962156816282</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>turn_L</t>
+        </is>
+      </c>
+      <c r="B68" t="n">
+        <v>0.4900533454460951</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>turn_M_b</t>
+        </is>
+      </c>
+      <c r="B69" t="n">
+        <v>1.463403371267119e-18</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>turn_M_g</t>
+        </is>
+      </c>
+      <c r="B70" t="n">
+        <v>-1.463403371267119e-18</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>turn_M_w</t>
+        </is>
+      </c>
+      <c r="B71" t="n">
+        <v>3.520786789153028e-19</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>turn_Y</t>
+        </is>
+      </c>
+      <c r="B72" t="n">
+        <v>2.617456789395252e-17</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>turn_fuselage_aero_components</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>[AeroComponentResults(
+	L=0.00011968880593709713,
+	Y=0.0,
+	D=0.0004967411139152521,
+	l_b=-0.0,
+	m_b=-5.357034034996522e-05,
+	n_b=-0.0,
+	span_effective=0.004055451774444796, oswalds_efficiency=0.95,
+)]</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>turn_l_b</t>
+        </is>
+      </c>
+      <c r="B74" t="n">
+        <v>1.463403371267119e-18</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>turn_m_b</t>
+        </is>
+      </c>
+      <c r="B75" t="n">
+        <v>0.00232707039471125</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>turn_n_b</t>
+        </is>
+      </c>
+      <c r="B76" t="n">
+        <v>-1.946716976662864e-17</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>turn_wing_aero_components</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>[AeroComponentResults(
+	L=0.4422075354169336,
+	Y=0.0,
+	D=0.03410682128253058,
+	l_b=-0.0,
+	m_b=0.03762132831443529,
+	n_b=-0.0,
+	span_effective=1.6206496155802028, oswalds_efficiency=0.7718502781381492,
+), AeroComponentResults(
+	L=0.04772612122322445,
+	Y=0.0,
+	D=0.0046365157976351636,
+	l_b=-0.0,
+	m_b=-0.03526246786689981,
+	n_b=-0.0,
+	span_effective=0.3593336687022275, oswalds_efficiency=0.8106853777008906,
+), AeroComponentResults(
+	L=1.3552527156068805e-20,
+	Y=2.6174567893952522e-17,
+	D=0.0016192108432932818,
+	l_b=1.4634033712671194e-18,
+	m_b=2.1780287525730196e-05,
+	n_b=-1.9467169766628638e-17,
+	span_effective=0.17111218630709724, oswalds_efficiency=0.8232692748986458,
+)]</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -2069,7 +2431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F27"/>
+  <dimension ref="A1:F32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2111,10 +2473,10 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.6874625936797452</v>
+        <v>0.8737940869410059</v>
       </c>
       <c r="C2" t="n">
-        <v>0.6874626036722987</v>
+        <v>0.8737940969317202</v>
       </c>
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="n">
@@ -2131,7 +2493,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.08111146596763252</v>
+        <v>0.07963424090427679</v>
       </c>
       <c r="C3" t="n">
         <v>0.001</v>
@@ -2147,11 +2509,11 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Trim Cm</t>
+          <t>Nominal Trim Cm</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>3.039702191125778e-14</v>
+        <v>-1.491448830018954e-10</v>
       </c>
       <c r="C4" t="n">
         <v>0</v>
@@ -2169,11 +2531,11 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Trim Cl</t>
+          <t>Nominal Trim Cl</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>9.30363791679246e-19</v>
+        <v>3.087405529260732e-19</v>
       </c>
       <c r="C5" t="n">
         <v>0</v>
@@ -2191,11 +2553,11 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Trim Cn</t>
+          <t>Nominal Trim Cn</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>-1.362037599096439e-17</v>
+        <v>-4.05887327666648e-18</v>
       </c>
       <c r="C6" t="n">
         <v>0</v>
@@ -2217,7 +2579,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.4783114757805177</v>
+        <v>0.3538598496885145</v>
       </c>
       <c r="C7" t="inlineStr"/>
       <c r="D7" t="n">
@@ -2233,15 +2595,15 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Alpha &lt;= stall margin</t>
+          <t>Alpha &lt;= turn stall margin</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>4.948056657649936</v>
+        <v>3.265624972678735</v>
       </c>
       <c r="C8" t="inlineStr"/>
       <c r="D8" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="E8" t="n">
         <v>1e-06</v>
@@ -2253,16 +2615,16 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>L/D minimum</t>
+          <t>Turn CL cap</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>8.475529143488501</v>
-      </c>
-      <c r="C9" t="n">
-        <v>8</v>
-      </c>
-      <c r="D9" t="inlineStr"/>
+        <v>0.3528117324472714</v>
+      </c>
+      <c r="C9" t="inlineStr"/>
+      <c r="D9" t="n">
+        <v>0.9</v>
+      </c>
       <c r="E9" t="n">
         <v>1e-06</v>
       </c>
@@ -2273,16 +2635,16 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Wing loading minimum</t>
+          <t>Turn footprint in width</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>4.687449300794357</v>
-      </c>
-      <c r="C10" t="n">
-        <v>2</v>
-      </c>
-      <c r="D10" t="inlineStr"/>
+        <v>2.080046038462513</v>
+      </c>
+      <c r="C10" t="inlineStr"/>
+      <c r="D10" t="n">
+        <v>2.4</v>
+      </c>
       <c r="E10" t="n">
         <v>1e-06</v>
       </c>
@@ -2293,16 +2655,16 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Wing loading maximum</t>
+          <t>L/D minimum</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>4.687449300794357</v>
-      </c>
-      <c r="C11" t="inlineStr"/>
-      <c r="D11" t="n">
-        <v>20</v>
-      </c>
+        <v>10.97259265635919</v>
+      </c>
+      <c r="C11" t="n">
+        <v>8</v>
+      </c>
+      <c r="D11" t="inlineStr"/>
       <c r="E11" t="n">
         <v>1e-06</v>
       </c>
@@ -2313,14 +2675,14 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Wing Reynolds</t>
+          <t>Wing loading minimum</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>39550.96498607255</v>
+        <v>3.467824177017998</v>
       </c>
       <c r="C12" t="n">
-        <v>20000</v>
+        <v>2</v>
       </c>
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="n">
@@ -2333,16 +2695,16 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Static margin minimum</t>
+          <t>Wing loading maximum</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.1000000099170008</v>
-      </c>
-      <c r="C13" t="n">
-        <v>0.05</v>
-      </c>
-      <c r="D13" t="inlineStr"/>
+        <v>3.467824177017998</v>
+      </c>
+      <c r="C13" t="inlineStr"/>
+      <c r="D13" t="n">
+        <v>20</v>
+      </c>
       <c r="E13" t="n">
         <v>1e-06</v>
       </c>
@@ -2353,16 +2715,16 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Static margin maximum</t>
+          <t>Wing Reynolds</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>0.1000000099170008</v>
-      </c>
-      <c r="C14" t="inlineStr"/>
-      <c r="D14" t="n">
-        <v>0.1</v>
-      </c>
+        <v>41933.23691995171</v>
+      </c>
+      <c r="C14" t="n">
+        <v>20000</v>
+      </c>
+      <c r="D14" t="inlineStr"/>
       <c r="E14" t="n">
         <v>1e-06</v>
       </c>
@@ -2373,14 +2735,14 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Vh minimum</t>
+          <t>Static margin minimum</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>0.4999999900541847</v>
+        <v>0.04999999020698476</v>
       </c>
       <c r="C15" t="n">
-        <v>0.5</v>
+        <v>0.05</v>
       </c>
       <c r="D15" t="inlineStr"/>
       <c r="E15" t="n">
@@ -2393,15 +2755,15 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Vh maximum</t>
+          <t>Static margin maximum</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>0.4999999900541847</v>
+        <v>0.04999999020698476</v>
       </c>
       <c r="C16" t="inlineStr"/>
       <c r="D16" t="n">
-        <v>0.7</v>
+        <v>0.1</v>
       </c>
       <c r="E16" t="n">
         <v>1e-06</v>
@@ -2413,14 +2775,14 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Vv minimum</t>
+          <t>Vh minimum</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>0.0500000099349265</v>
+        <v>0.7000000080815174</v>
       </c>
       <c r="C17" t="n">
-        <v>0.03</v>
+        <v>0.5</v>
       </c>
       <c r="D17" t="inlineStr"/>
       <c r="E17" t="n">
@@ -2433,15 +2795,15 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Vv maximum</t>
+          <t>Vh maximum</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>0.0500000099349265</v>
+        <v>0.7000000080815174</v>
       </c>
       <c r="C18" t="inlineStr"/>
       <c r="D18" t="n">
-        <v>0.05</v>
+        <v>0.7</v>
       </c>
       <c r="E18" t="n">
         <v>1e-06</v>
@@ -2453,16 +2815,16 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Clb &lt;= 0</t>
+          <t>Vv minimum</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>-0.2439029982603689</v>
-      </c>
-      <c r="C19" t="inlineStr"/>
-      <c r="D19" t="n">
-        <v>0</v>
-      </c>
+        <v>0.02999999000825085</v>
+      </c>
+      <c r="C19" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="D19" t="inlineStr"/>
       <c r="E19" t="n">
         <v>1e-06</v>
       </c>
@@ -2473,16 +2835,16 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Cnb &gt;= 0</t>
+          <t>Vv maximum</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>0.09957879373723921</v>
-      </c>
-      <c r="C20" t="n">
-        <v>0</v>
-      </c>
-      <c r="D20" t="inlineStr"/>
+        <v>0.02999999000825085</v>
+      </c>
+      <c r="C20" t="inlineStr"/>
+      <c r="D20" t="n">
+        <v>0.05</v>
+      </c>
       <c r="E20" t="n">
         <v>1e-06</v>
       </c>
@@ -2493,15 +2855,15 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Cmq &lt;= -0.01</t>
+          <t>Clb &lt;= 0</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>-29.3329799057312</v>
+        <v>-0.2819421253289612</v>
       </c>
       <c r="C21" t="inlineStr"/>
       <c r="D21" t="n">
-        <v>-0.01</v>
+        <v>0</v>
       </c>
       <c r="E21" t="n">
         <v>1e-06</v>
@@ -2513,14 +2875,14 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Roll rate minimum</t>
+          <t>Cnb &gt;= 0</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>0.9369224915803962</v>
+        <v>0.03795793197254786</v>
       </c>
       <c r="C22" t="n">
-        <v>0.6</v>
+        <v>0</v>
       </c>
       <c r="D22" t="inlineStr"/>
       <c r="E22" t="n">
@@ -2533,16 +2895,16 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Roll accel minimum</t>
+          <t>Cmq &lt;= -0.01</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>86.48660579196596</v>
-      </c>
-      <c r="C23" t="n">
-        <v>2</v>
-      </c>
-      <c r="D23" t="inlineStr"/>
+        <v>-39.52415518558014</v>
+      </c>
+      <c r="C23" t="inlineStr"/>
+      <c r="D23" t="n">
+        <v>-0.01</v>
+      </c>
       <c r="E23" t="n">
         <v>1e-06</v>
       </c>
@@ -2553,16 +2915,16 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Roll time constant</t>
+          <t>Roll rate minimum</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>0.01083315136489528</v>
-      </c>
-      <c r="C24" t="inlineStr"/>
-      <c r="D24" t="n">
-        <v>0.45</v>
-      </c>
+        <v>0.5999999902481539</v>
+      </c>
+      <c r="C24" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="D24" t="inlineStr"/>
       <c r="E24" t="n">
         <v>1e-06</v>
       </c>
@@ -2573,16 +2935,16 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Aileron servo torque</t>
+          <t>Roll accel minimum</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>4.260761353003889e-06</v>
-      </c>
-      <c r="C25" t="inlineStr"/>
-      <c r="D25" t="n">
-        <v>0.144</v>
-      </c>
+        <v>64.60823526290454</v>
+      </c>
+      <c r="C25" t="n">
+        <v>2</v>
+      </c>
+      <c r="D25" t="inlineStr"/>
       <c r="E25" t="n">
         <v>1e-06</v>
       </c>
@@ -2593,15 +2955,15 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Elevator servo torque</t>
+          <t>Roll time constant</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>4.729757469507889e-08</v>
+        <v>0.009286741663916792</v>
       </c>
       <c r="C26" t="inlineStr"/>
       <c r="D26" t="n">
-        <v>0.144</v>
+        <v>0.45</v>
       </c>
       <c r="E26" t="n">
         <v>1e-06</v>
@@ -2613,11 +2975,11 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Rudder servo torque</t>
+          <t>Aileron servo torque</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>4.924150186828811e-22</v>
+        <v>7.761185342964752e-06</v>
       </c>
       <c r="C27" t="inlineStr"/>
       <c r="D27" t="n">
@@ -2628,6 +2990,542 @@
       </c>
       <c r="F27" t="b">
         <v>1</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Elevator servo torque</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>1.628272149107434e-07</v>
+      </c>
+      <c r="C28" t="inlineStr"/>
+      <c r="D28" t="n">
+        <v>0.144</v>
+      </c>
+      <c r="E28" t="n">
+        <v>1e-06</v>
+      </c>
+      <c r="F28" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Rudder servo torque</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>1.358258982162884e-22</v>
+      </c>
+      <c r="C29" t="inlineStr"/>
+      <c r="D29" t="n">
+        <v>0.144</v>
+      </c>
+      <c r="E29" t="n">
+        <v>1e-06</v>
+      </c>
+      <c r="F29" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Turn aileron trim utilization</t>
+        </is>
+      </c>
+      <c r="B30" t="n">
+        <v>1.732786463659694e-16</v>
+      </c>
+      <c r="C30" t="inlineStr"/>
+      <c r="D30" t="n">
+        <v>24</v>
+      </c>
+      <c r="E30" t="n">
+        <v>1e-06</v>
+      </c>
+      <c r="F30" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Turn elevator trim utilization</t>
+        </is>
+      </c>
+      <c r="B31" t="n">
+        <v>0.7295201394751571</v>
+      </c>
+      <c r="C31" t="inlineStr"/>
+      <c r="D31" t="n">
+        <v>24</v>
+      </c>
+      <c r="E31" t="n">
+        <v>1e-06</v>
+      </c>
+      <c r="F31" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Turn rudder trim utilization</t>
+        </is>
+      </c>
+      <c r="B32" t="n">
+        <v>1.035118855641136e-15</v>
+      </c>
+      <c r="C32" t="inlineStr"/>
+      <c r="D32" t="n">
+        <v>24</v>
+      </c>
+      <c r="E32" t="n">
+        <v>1e-06</v>
+      </c>
+      <c r="F32" t="b">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D21"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>DesignPoint</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Metric</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Unit</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Settings</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>V_NOM_MPS</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>4</v>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>m/s</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Settings</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>V_TURN_MPS</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>3</v>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>m/s</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Settings</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>TURN_BANK_DEG</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>50</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>deg</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Settings</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>WALL_CLEARANCE_M</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Arena</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>ARENA_LENGTH_M</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>8.4</v>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Arena</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>ARENA_WIDTH_M</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Arena</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>ARENA_HEIGHT_M</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Nominal</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>alpha_nom_deg</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>3.265624972678735</v>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>deg</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Nominal</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>delta_a_nom_deg</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>1.732786463659694e-16</v>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>deg</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Nominal</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>delta_e_nom_deg</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>0.7295201394751571</v>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>deg</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Nominal</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>delta_r_nom_deg</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>1.035118855641136e-15</v>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>deg</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Nominal</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>sink_nom_mps</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>0.3645446504338175</v>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>m/s</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Nominal</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>CL_nom</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>0.3538598496885145</v>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Manoeuvre</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>alpha_turn_deg</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>3.265624972678735</v>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>deg</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Manoeuvre</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>delta_a_turn_deg</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>1.732786463659694e-16</v>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>deg</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Manoeuvre</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>delta_e_turn_deg</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>0.7295201394751571</v>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>deg</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Manoeuvre</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>delta_r_turn_deg</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>1.035118855641136e-15</v>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>deg</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Manoeuvre</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>CL_turn</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>0.3528117324472714</v>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Manoeuvre</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>turn_radius_m</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>0.769816175392</v>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Manoeuvre</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>turn_footprint_lhs_m</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>2.080046038462513</v>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
- Python - Lift to drag ratio penalty - Rename the structure, make it proxy not deflection
</commit_message>
<xml_diff>
--- a/02_Glider_Design/C_results/nausicaa_results.xlsx
+++ b/02_Glider_Design/C_results/nausicaa_results.xlsx
@@ -459,7 +459,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>bdcac3f-dirty</t>
+          <t>3f20d9c-dirty</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -492,7 +492,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>225.7690647637066</v>
+        <v>126.7317013672611</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -507,7 +507,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>4.5</v>
+        <v>4.7</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -522,7 +522,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>4.1</v>
+        <v>4.2</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -597,7 +597,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.6440573443182428</v>
+        <v>0.6399411649061671</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
@@ -612,7 +612,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.5340573443182428</v>
+        <v>0.5299411649061672</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -627,7 +627,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.6440573443182428</v>
+        <v>0.6399411649061671</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
@@ -642,7 +642,7 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>4.995818923191007</v>
+        <v>5.121658855088541</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
@@ -657,7 +657,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>2.318821944480995e-16</v>
+        <v>-1.003039419388021e-16</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
@@ -672,7 +672,7 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>1.248382770292376</v>
+        <v>1.07084831044651</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
@@ -687,7 +687,7 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>3.758299667982743e-15</v>
+        <v>7.417831106112554e-15</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
@@ -702,7 +702,7 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>8.000000079995392</v>
+        <v>7.608325391688213</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
@@ -717,7 +717,7 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>-2.809137900571732e-18</v>
+        <v>5.377062767205443e-18</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
@@ -732,7 +732,7 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>4.149054262853123</v>
+        <v>8.219893660890538</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
@@ -747,7 +747,7 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>7.814204555748593e-17</v>
+        <v>1.454124360923813e-15</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
@@ -762,7 +762,7 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>0.1070485325235647</v>
+        <v>0.08976216479594404</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
@@ -777,7 +777,7 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>107.0485325235647</v>
+        <v>89.76216479594405</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
@@ -792,7 +792,7 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>0.2360016164371651</v>
+        <v>0.197891699095256</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
@@ -822,7 +822,7 @@
         </is>
       </c>
       <c r="B26" t="n">
-        <v>0.6766792150473272</v>
+        <v>0.739374410448861</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
@@ -837,7 +837,7 @@
         </is>
       </c>
       <c r="B27" t="n">
-        <v>0.05787929025254737</v>
+        <v>0.05287817641095208</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
@@ -852,7 +852,7 @@
         </is>
       </c>
       <c r="B28" t="n">
-        <v>0.617381854787086</v>
+        <v>0.5874999992029738</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
@@ -867,7 +867,7 @@
         </is>
       </c>
       <c r="B29" t="n">
-        <v>7.999999920130635</v>
+        <v>7.999999920010524</v>
       </c>
       <c r="C29" t="inlineStr">
         <is>
@@ -882,7 +882,7 @@
         </is>
       </c>
       <c r="B30" t="n">
-        <v>1.437845545371058</v>
+        <v>1.50883970376832</v>
       </c>
       <c r="C30" t="inlineStr">
         <is>
@@ -897,7 +897,7 @@
         </is>
       </c>
       <c r="B31" t="n">
-        <v>2.393570521135981</v>
+        <v>2.400000023994921</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
@@ -912,7 +912,7 @@
         </is>
       </c>
       <c r="B32" t="n">
-        <v>0.7071245061333374</v>
+        <v>0.6677777267646771</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
@@ -927,7 +927,7 @@
         </is>
       </c>
       <c r="B33" t="n">
-        <v>5.199892746342704</v>
+        <v>6.333919194811074</v>
       </c>
       <c r="C33" t="inlineStr">
         <is>
@@ -942,7 +942,7 @@
         </is>
       </c>
       <c r="B34" t="n">
-        <v>67223.26919679661</v>
+        <v>56310.25292766299</v>
       </c>
       <c r="C34" t="inlineStr">
         <is>
@@ -957,7 +957,7 @@
         </is>
       </c>
       <c r="B35" t="n">
-        <v>0.04999998999434588</v>
+        <v>0.04999999007341833</v>
       </c>
       <c r="C35" t="inlineStr">
         <is>
@@ -972,7 +972,7 @@
         </is>
       </c>
       <c r="B36" t="n">
-        <v>0.4999999900064669</v>
+        <v>0.4999999900054579</v>
       </c>
       <c r="C36" t="inlineStr">
         <is>
@@ -987,7 +987,7 @@
         </is>
       </c>
       <c r="B37" t="n">
-        <v>0.02999999000058427</v>
+        <v>0.02999999000124711</v>
       </c>
       <c r="C37" t="inlineStr">
         <is>
@@ -1002,7 +1002,7 @@
         </is>
       </c>
       <c r="B38" t="n">
-        <v>4.065798068775985</v>
+        <v>4.778401783804584</v>
       </c>
       <c r="C38" t="inlineStr">
         <is>
@@ -1017,7 +1017,7 @@
         </is>
       </c>
       <c r="B39" t="n">
-        <v>3.704393795995896</v>
+        <v>4.270061168506224</v>
       </c>
       <c r="C39" t="inlineStr">
         <is>
@@ -1047,7 +1047,7 @@
         </is>
       </c>
       <c r="B41" t="n">
-        <v>162.8965872304802</v>
+        <v>206.9382837941339</v>
       </c>
       <c r="C41" t="inlineStr">
         <is>
@@ -1062,7 +1062,7 @@
         </is>
       </c>
       <c r="B42" t="n">
-        <v>0.02495938151867688</v>
+        <v>0.02309095106132333</v>
       </c>
       <c r="C42" t="inlineStr">
         <is>
@@ -1073,11 +1073,11 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>wing_tip_deflection_m</t>
+          <t>wing_tip_deflection_proxy_m</t>
         </is>
       </c>
       <c r="B43" t="n">
-        <v>1.640336697806695</v>
+        <v>1.084473598671871</v>
       </c>
       <c r="C43" t="inlineStr">
         <is>
@@ -1088,11 +1088,11 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>wing_tip_deflection_allow_m</t>
+          <t>wing_tip_deflection_proxy_allow_m</t>
         </is>
       </c>
       <c r="B44" t="n">
-        <v>0.03645799806119386</v>
+        <v>0.03129282561812807</v>
       </c>
       <c r="C44" t="inlineStr">
         <is>
@@ -1103,11 +1103,11 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>wing_tip_deflection_semispan_fraction</t>
+          <t>wing_tip_deflection_proxy_semispan_fraction</t>
         </is>
       </c>
       <c r="B45" t="n">
-        <v>3.599400482831624</v>
+        <v>2.772452988185589</v>
       </c>
       <c r="C45" t="inlineStr">
         <is>
@@ -1118,11 +1118,11 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>wing_tip_deflection_over_allow</t>
+          <t>wing_tip_deflection_proxy_over_allow</t>
         </is>
       </c>
       <c r="B46" t="n">
-        <v>44.9925060353953</v>
+        <v>34.65566235231987</v>
       </c>
       <c r="C46" t="inlineStr">
         <is>
@@ -1137,7 +1137,7 @@
         </is>
       </c>
       <c r="B47" t="n">
-        <v>0.4627552680926893</v>
+        <v>0.3971945986718404</v>
       </c>
       <c r="C47" t="inlineStr">
         <is>
@@ -1152,7 +1152,7 @@
         </is>
       </c>
       <c r="B48" t="n">
-        <v>0.8168686578824084</v>
+        <v>0.6849594044583612</v>
       </c>
       <c r="C48" t="inlineStr">
         <is>
@@ -1167,7 +1167,7 @@
         </is>
       </c>
       <c r="B49" t="n">
-        <v>1.765228219333401</v>
+        <v>1.724493250282767</v>
       </c>
       <c r="C49" t="inlineStr">
         <is>
@@ -1208,11 +1208,11 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>htail_tip_deflection_m</t>
+          <t>htail_tip_deflection_proxy_m</t>
         </is>
       </c>
       <c r="B52" t="n">
-        <v>0.8605320307455027</v>
+        <v>0.4929079927997522</v>
       </c>
       <c r="C52" t="inlineStr">
         <is>
@@ -1223,11 +1223,11 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>htail_tip_deflection_allow_m</t>
+          <t>htail_tip_deflection_proxy_allow_m</t>
         </is>
       </c>
       <c r="B53" t="n">
-        <v>0.01665499913439414</v>
+        <v>0.01287631970508052</v>
       </c>
       <c r="C53" t="inlineStr">
         <is>
@@ -1238,11 +1238,11 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>htail_tip_deflection_semispan_fraction</t>
+          <t>htail_tip_deflection_proxy_semispan_fraction</t>
         </is>
       </c>
       <c r="B54" t="n">
-        <v>4.133447375417382</v>
+        <v>3.062415373891464</v>
       </c>
       <c r="C54" t="inlineStr">
         <is>
@@ -1253,11 +1253,11 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>htail_tip_deflection_over_allow</t>
+          <t>htail_tip_deflection_proxy_over_allow</t>
         </is>
       </c>
       <c r="B55" t="n">
-        <v>51.66809219271727</v>
+        <v>38.28019217364329</v>
       </c>
       <c r="C55" t="inlineStr">
         <is>
@@ -1272,7 +1272,7 @@
         </is>
       </c>
       <c r="B56" t="n">
-        <v>0.2081874891799267</v>
+        <v>0.1609539963135065</v>
       </c>
       <c r="C56" t="inlineStr">
         <is>
@@ -1287,7 +1287,7 @@
         </is>
       </c>
       <c r="B57" t="n">
-        <v>0.2042171644706021</v>
+        <v>0.1712398511145903</v>
       </c>
       <c r="C57" t="inlineStr">
         <is>
@@ -1302,7 +1302,7 @@
         </is>
       </c>
       <c r="B58" t="n">
-        <v>0.9809290907683061</v>
+        <v>1.063905557095016</v>
       </c>
       <c r="C58" t="inlineStr">
         <is>
@@ -1343,11 +1343,11 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>objective_struct_deflection_penalty</t>
+          <t>objective_struct_deflection_proxy_penalty</t>
         </is>
       </c>
       <c r="B61" t="n">
-        <v>96.7670293637146</v>
+        <v>56.63518041868387</v>
       </c>
       <c r="C61" t="inlineStr">
         <is>
@@ -1358,11 +1358,11 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>objective_htail_deflection_penalty</t>
+          <t>objective_htail_deflection_proxy_penalty</t>
         </is>
       </c>
       <c r="B62" t="n">
-        <v>128.3627783308596</v>
+        <v>69.49070752484344</v>
       </c>
       <c r="C62" t="inlineStr">
         <is>
@@ -1377,7 +1377,7 @@
         </is>
       </c>
       <c r="B63" t="n">
-        <v>0.0001538199322950294</v>
+        <v>0.0001316523508435627</v>
       </c>
       <c r="C63" t="inlineStr">
         <is>
@@ -1392,7 +1392,7 @@
         </is>
       </c>
       <c r="B64" t="n">
-        <v>0.003577412893454938</v>
+        <v>0.002154550749008229</v>
       </c>
       <c r="C64" t="inlineStr">
         <is>
@@ -1407,7 +1407,7 @@
         </is>
       </c>
       <c r="B65" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C65" t="inlineStr">
         <is>
@@ -1423,7 +1423,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>alpha_turn_deg:upper; ballast_mass_kg:lower</t>
+          <t>ballast_mass_kg:lower</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
@@ -1470,7 +1470,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.9255105361853786</v>
+        <v>0.7943891973436807</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -1485,7 +1485,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.2182096598924276</v>
+        <v>0.1750074259201051</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -1500,7 +1500,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.2019553393278698</v>
+        <v>0.139024008605856</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -1515,7 +1515,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>4.241382057245469</v>
+        <v>4.539174227420141</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -1530,7 +1530,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.6440573443182428</v>
+        <v>0.6399411649061671</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -1545,7 +1545,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.5340573443182428</v>
+        <v>0.5299411649061672</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -1560,7 +1560,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0.6440573443182428</v>
+        <v>0.6399411649061671</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -1575,7 +1575,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>0.4163749783598534</v>
+        <v>0.321907992627013</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
@@ -1590,7 +1590,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>0.1189642795313867</v>
+        <v>0.08047699815675324</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
@@ -1605,7 +1605,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.04953374931547669</v>
+        <v>0.02590618892928826</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
@@ -1620,7 +1620,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.1575689288959599</v>
+        <v>0.1178844373525108</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -1635,7 +1635,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.07878446444797996</v>
+        <v>0.05894221867625538</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
@@ -1650,7 +1650,7 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>0.01241398367671004</v>
+        <v>0.006948370284959018</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
@@ -1786,28 +1786,28 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.03998715718691821</v>
+        <v>0.02752675370395948</v>
       </c>
       <c r="C2" t="n">
-        <v>39.98715718691821</v>
+        <v>27.52675370395948</v>
       </c>
       <c r="D2" t="n">
-        <v>0.1091048299462138</v>
+        <v>0.08750371296005256</v>
       </c>
       <c r="E2" t="n">
         <v>0</v>
       </c>
       <c r="F2" t="n">
-        <v>0.04017830450503364</v>
+        <v>0.03448605911925642</v>
       </c>
       <c r="G2" t="n">
-        <v>0.002768367587653758</v>
+        <v>0.001404005707300966</v>
       </c>
       <c r="H2" t="n">
-        <v>0.0001637203424472442</v>
+        <v>7.252347189887447e-05</v>
       </c>
       <c r="I2" t="n">
-        <v>0.00293184800715788</v>
+        <v>0.001476364018677616</v>
       </c>
     </row>
     <row r="3">
@@ -1823,7 +1823,7 @@
         <v>9</v>
       </c>
       <c r="D3" t="n">
-        <v>0.05787929025254737</v>
+        <v>0.05287817641095208</v>
       </c>
       <c r="E3" t="n">
         <v>0</v>
@@ -1848,13 +1848,13 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.008498136449883124</v>
+        <v>0.008443824742075418</v>
       </c>
       <c r="C4" t="n">
-        <v>8.498136449883123</v>
+        <v>8.443824742075417</v>
       </c>
       <c r="D4" t="n">
-        <v>0.2120286721591214</v>
+        <v>0.2099705824530836</v>
       </c>
       <c r="E4" t="n">
         <v>0</v>
@@ -1879,44 +1879,44 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.007929520927671456</v>
+        <v>0.006649049244144003</v>
       </c>
       <c r="C5" t="n">
-        <v>7.929520927671456</v>
+        <v>6.649049244144003</v>
       </c>
       <c r="D5" t="n">
-        <v>0.1469015240633527</v>
+        <v>0.127347442746731</v>
       </c>
       <c r="E5" t="n">
         <v>0</v>
       </c>
       <c r="F5" t="n">
-        <v>0.01899822970330011</v>
+        <v>0.0136560917668209</v>
       </c>
       <c r="G5" t="n">
-        <v>0.0002468923347374914</v>
+        <v>0.0001274016940968726</v>
       </c>
       <c r="H5" t="n">
-        <v>0.0001552806533449748</v>
+        <v>0.0001207184376797192</v>
       </c>
       <c r="I5" t="n">
-        <v>0.0003946558443010751</v>
+        <v>0.0002440523717955666</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>htail_surfaces</t>
+          <t>flight_controller</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.005944049917857202</v>
+        <v>0.005</v>
       </c>
       <c r="C6" t="n">
-        <v>5.944049917857202</v>
+        <v>5</v>
       </c>
       <c r="D6" t="n">
-        <v>0.5043162744353962</v>
+        <v>0.06787817641095208</v>
       </c>
       <c r="E6" t="n">
         <v>0</v>
@@ -1925,19 +1925,19 @@
         <v>0</v>
       </c>
       <c r="G6" t="n">
-        <v>8.588018928113547e-05</v>
+        <v>0</v>
       </c>
       <c r="H6" t="n">
-        <v>7.014721812434071e-06</v>
+        <v>0</v>
       </c>
       <c r="I6" t="n">
-        <v>9.288599501869274e-05</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>flight_controller</t>
+          <t>receiver</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -1947,7 +1947,7 @@
         <v>5</v>
       </c>
       <c r="D7" t="n">
-        <v>0.07287929025254737</v>
+        <v>0.07287817641095208</v>
       </c>
       <c r="E7" t="n">
         <v>0</v>
@@ -1968,17 +1968,17 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>receiver</t>
+          <t>tail mount module 1</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0.005</v>
+        <v>0.004</v>
       </c>
       <c r="C8" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D8" t="n">
-        <v>0.07787929025254738</v>
+        <v>0.4937265157356281</v>
       </c>
       <c r="E8" t="n">
         <v>0</v>
@@ -1999,7 +1999,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>tail mount module 1</t>
+          <t>avionics tray</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -2009,7 +2009,7 @@
         <v>4</v>
       </c>
       <c r="D9" t="n">
-        <v>0.4805234185291188</v>
+        <v>0.05250222777603154</v>
       </c>
       <c r="E9" t="n">
         <v>0</v>
@@ -2030,17 +2030,17 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>avionics tray</t>
+          <t>htail_surfaces</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>0.004</v>
+        <v>0.003108742671514591</v>
       </c>
       <c r="C10" t="n">
-        <v>4</v>
+        <v>3.108742671514591</v>
       </c>
       <c r="D10" t="n">
-        <v>0.06546289796772828</v>
+        <v>0.5098219153669787</v>
       </c>
       <c r="E10" t="n">
         <v>0</v>
@@ -2049,13 +2049,13 @@
         <v>0</v>
       </c>
       <c r="G10" t="n">
-        <v>0</v>
+        <v>2.684755655060274e-05</v>
       </c>
       <c r="H10" t="n">
-        <v>0</v>
+        <v>1.68015811910358e-06</v>
       </c>
       <c r="I10" t="n">
-        <v>0</v>
+        <v>2.852305155569905e-05</v>
       </c>
     </row>
     <row r="11">
@@ -2071,7 +2071,7 @@
         <v>3</v>
       </c>
       <c r="D11" t="n">
-        <v>0.06546289796772828</v>
+        <v>0.05250222777603154</v>
       </c>
       <c r="E11" t="n">
         <v>0</v>
@@ -2102,7 +2102,7 @@
         <v>3</v>
       </c>
       <c r="D12" t="n">
-        <v>0.06546289796772828</v>
+        <v>0.05250222777603154</v>
       </c>
       <c r="E12" t="n">
         <v>0</v>
@@ -2133,7 +2133,7 @@
         <v>2.2</v>
       </c>
       <c r="D13" t="n">
-        <v>0.06546289796772828</v>
+        <v>0.05250222777603154</v>
       </c>
       <c r="E13" t="n">
         <v>0</v>
@@ -2164,7 +2164,7 @@
         <v>2.2</v>
       </c>
       <c r="D14" t="n">
-        <v>0.06546289796772828</v>
+        <v>0.05250222777603154</v>
       </c>
       <c r="E14" t="n">
         <v>0</v>
@@ -2195,13 +2195,13 @@
         <v>2.2</v>
       </c>
       <c r="D15" t="n">
-        <v>0.06546289796772828</v>
+        <v>0.05250222777603154</v>
       </c>
       <c r="E15" t="n">
-        <v>0.2050762390942155</v>
+        <v>0.1760221441019704</v>
       </c>
       <c r="F15" t="n">
-        <v>0.03616047405453028</v>
+        <v>0.03103745320733078</v>
       </c>
       <c r="G15" t="n">
         <v>0</v>
@@ -2226,13 +2226,13 @@
         <v>2.2</v>
       </c>
       <c r="D16" t="n">
-        <v>0.06546289796772828</v>
+        <v>0.05250222777603154</v>
       </c>
       <c r="E16" t="n">
-        <v>-0.2050762390942155</v>
+        <v>-0.1760221441019704</v>
       </c>
       <c r="F16" t="n">
-        <v>0.03616047405453028</v>
+        <v>0.03103745320733078</v>
       </c>
       <c r="G16" t="n">
         <v>0</v>
@@ -2247,63 +2247,63 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>vtail_surfaces</t>
+          <t>linkages</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>0.001489678041205204</v>
+        <v>0.001</v>
       </c>
       <c r="C17" t="n">
-        <v>1.489678041205204</v>
+        <v>1</v>
       </c>
       <c r="D17" t="n">
-        <v>0.4842263668936928</v>
+        <v>0.2347917081443011</v>
       </c>
       <c r="E17" t="n">
         <v>0</v>
       </c>
       <c r="F17" t="n">
-        <v>0.07878446444797996</v>
+        <v>0</v>
       </c>
       <c r="G17" t="n">
-        <v>3.083257073043368e-06</v>
+        <v>0</v>
       </c>
       <c r="H17" t="n">
-        <v>3.85267476814058e-06</v>
+        <v>0</v>
       </c>
       <c r="I17" t="n">
-        <v>7.7165221215902e-07</v>
+        <v>0</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>linkages</t>
+          <t>vtail_surfaces</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>0.001</v>
+        <v>0.0008338044341950822</v>
       </c>
       <c r="C18" t="n">
-        <v>1</v>
+        <v>0.8338044341950822</v>
       </c>
       <c r="D18" t="n">
-        <v>0.2224170673348514</v>
+        <v>0.4990545256267299</v>
       </c>
       <c r="E18" t="n">
         <v>0</v>
       </c>
       <c r="F18" t="n">
-        <v>0</v>
+        <v>0.05894221867625538</v>
       </c>
       <c r="G18" t="n">
-        <v>0</v>
+        <v>9.662223456636757e-07</v>
       </c>
       <c r="H18" t="n">
-        <v>0</v>
+        <v>1.206996240422537e-06</v>
       </c>
       <c r="I18" t="n">
-        <v>0</v>
+        <v>2.420246014101536e-07</v>
       </c>
     </row>
     <row r="19">
@@ -2319,7 +2319,7 @@
         <v>0.4</v>
       </c>
       <c r="D19" t="n">
-        <v>0.06787929025254737</v>
+        <v>0.06287817641095207</v>
       </c>
       <c r="E19" t="n">
         <v>0</v>
@@ -2344,13 +2344,13 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>-9.999970538854929e-09</v>
+        <v>-9.99994450676177e-09</v>
       </c>
       <c r="C20" t="n">
-        <v>-9.999970538854929e-06</v>
+        <v>-9.99994450676177e-06</v>
       </c>
       <c r="D20" t="n">
-        <v>0.06546289796772828</v>
+        <v>0.05250222777603154</v>
       </c>
       <c r="E20" t="n">
         <v>0</v>
@@ -2401,7 +2401,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.05751815038676538</v>
+        <v>0.0585168609929957</v>
       </c>
     </row>
     <row r="3">
@@ -2411,7 +2411,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>1.152405761619146</v>
+        <v>1.201985309532947</v>
       </c>
     </row>
     <row r="4">
@@ -2421,7 +2421,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>1.073697533394615e-05</v>
+        <v>1.328843061191225e-05</v>
       </c>
     </row>
     <row r="5">
@@ -2431,7 +2431,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.005419148698872222</v>
+        <v>0.007000042905977444</v>
       </c>
     </row>
     <row r="6">
@@ -2441,7 +2441,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.1337423730331383</v>
+        <v>-0.1004116753205303</v>
       </c>
     </row>
     <row r="7">
@@ -2451,7 +2451,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>7.472239453576446e-05</v>
+        <v>9.356877442301405e-05</v>
       </c>
     </row>
     <row r="8">
@@ -2461,7 +2461,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0.4601451985001849</v>
+        <v>0.4681348832632325</v>
       </c>
     </row>
     <row r="9">
@@ -2471,7 +2471,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>4.205442473775639</v>
+        <v>4.277116033625902</v>
       </c>
     </row>
     <row r="10">
@@ -2481,7 +2481,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>-8.942361667426424e-06</v>
+        <v>-3.594293956647017e-06</v>
       </c>
     </row>
     <row r="11">
@@ -2491,7 +2491,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>-0.004376802865635465</v>
+        <v>-0.001640654347379034</v>
       </c>
     </row>
     <row r="12">
@@ -2501,7 +2501,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.1663165750367956</v>
+        <v>-0.1829936964112822</v>
       </c>
     </row>
     <row r="13">
@@ -2511,7 +2511,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>-8.509891452623819e-05</v>
+        <v>-1.599603727253651e-05</v>
       </c>
     </row>
     <row r="14">
@@ -2521,7 +2521,7 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>-1.424111831562682e-17</v>
+        <v>-4.515946520211539e-17</v>
       </c>
     </row>
     <row r="15">
@@ -2531,7 +2531,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>2.064475784849059e-22</v>
+        <v>7.319503129305733e-22</v>
       </c>
     </row>
     <row r="16">
@@ -2541,7 +2541,7 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>-0.2011796791725537</v>
+        <v>-0.1817904219295661</v>
       </c>
     </row>
     <row r="17">
@@ -2551,7 +2551,7 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>-0.3023435725556479</v>
+        <v>-0.3205136839584692</v>
       </c>
     </row>
     <row r="18">
@@ -2561,7 +2561,7 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>8.317272200571798e-18</v>
+        <v>1.325508940677575e-17</v>
       </c>
     </row>
     <row r="19">
@@ -2571,7 +2571,7 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>0.1129973019841508</v>
+        <v>0.1187186584023332</v>
       </c>
     </row>
     <row r="20">
@@ -2581,7 +2581,7 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>-9.400956093217906e-19</v>
+        <v>-2.574427574422738e-18</v>
       </c>
     </row>
     <row r="21">
@@ -2591,7 +2591,7 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>-2.304523668986025e-19</v>
+        <v>3.916820998576346e-23</v>
       </c>
     </row>
     <row r="22">
@@ -2601,7 +2601,7 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>-0.1497243077168116</v>
+        <v>-0.1588441682609945</v>
       </c>
     </row>
     <row r="23">
@@ -2611,7 +2611,7 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>-0.5775611233947082</v>
+        <v>-0.6081823484123782</v>
       </c>
     </row>
     <row r="24">
@@ -2621,7 +2621,7 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>4.453099110204681e-19</v>
+        <v>2.159926378475337e-18</v>
       </c>
     </row>
     <row r="25">
@@ -2631,7 +2631,7 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>0.04978841957870687</v>
+        <v>0.0469233778768687</v>
       </c>
     </row>
     <row r="26">
@@ -2641,7 +2641,7 @@
         </is>
       </c>
       <c r="B26" t="n">
-        <v>4.321499743788634e-15</v>
+        <v>5.47347271698509e-14</v>
       </c>
     </row>
     <row r="27">
@@ -2651,7 +2651,7 @@
         </is>
       </c>
       <c r="B27" t="n">
-        <v>-0.2102720816105791</v>
+        <v>-0.2138557592241535</v>
       </c>
     </row>
     <row r="28">
@@ -2661,7 +2661,7 @@
         </is>
       </c>
       <c r="B28" t="n">
-        <v>-5.239409296253893e-06</v>
+        <v>-2.744099530098935e-06</v>
       </c>
     </row>
     <row r="29">
@@ -2671,7 +2671,7 @@
         </is>
       </c>
       <c r="B29" t="n">
-        <v>-0.0020621132823843</v>
+        <v>0.0007723394382532205</v>
       </c>
     </row>
     <row r="30">
@@ -2681,7 +2681,7 @@
         </is>
       </c>
       <c r="B30" t="n">
-        <v>-6.231079381770853</v>
+        <v>-9.078162866799115</v>
       </c>
     </row>
     <row r="31">
@@ -2691,7 +2691,7 @@
         </is>
       </c>
       <c r="B31" t="n">
-        <v>-0.0001217899959902428</v>
+        <v>-0.0001277220925384723</v>
       </c>
     </row>
     <row r="32">
@@ -2701,7 +2701,7 @@
         </is>
       </c>
       <c r="B32" t="n">
-        <v>5.041479338892034e-18</v>
+        <v>2.008185553909865e-17</v>
       </c>
     </row>
     <row r="33">
@@ -2711,7 +2711,7 @@
         </is>
       </c>
       <c r="B33" t="n">
-        <v>-2.02213262557967e-20</v>
+        <v>-3.257187420208019e-22</v>
       </c>
     </row>
     <row r="34">
@@ -2721,7 +2721,7 @@
         </is>
       </c>
       <c r="B34" t="n">
-        <v>0.03505599997496323</v>
+        <v>0.0407860197448539</v>
       </c>
     </row>
     <row r="35">
@@ -2731,7 +2731,7 @@
         </is>
       </c>
       <c r="B35" t="n">
-        <v>-0.03421589833381396</v>
+        <v>-0.02682529655707725</v>
       </c>
     </row>
     <row r="36">
@@ -2741,7 +2741,7 @@
         </is>
       </c>
       <c r="B36" t="n">
-        <v>-3.003814999326735e-18</v>
+        <v>-5.89437524336239e-18</v>
       </c>
     </row>
     <row r="37">
@@ -2751,7 +2751,7 @@
         </is>
       </c>
       <c r="B37" t="n">
-        <v>-0.03028335527322533</v>
+        <v>-0.04198303977746306</v>
       </c>
     </row>
     <row r="38">
@@ -2761,7 +2761,7 @@
         </is>
       </c>
       <c r="B38" t="n">
-        <v>0.1440758110043622</v>
+        <v>0.1100708544316998</v>
       </c>
     </row>
     <row r="39">
@@ -2771,7 +2771,7 @@
         </is>
       </c>
       <c r="B39" t="n">
-        <v>0.05068158451746413</v>
+        <v>0.03689004728669686</v>
       </c>
     </row>
     <row r="40">
@@ -2781,7 +2781,7 @@
         </is>
       </c>
       <c r="B40" t="n">
-        <v>0.0933942264868981</v>
+        <v>0.07318080714500298</v>
       </c>
     </row>
     <row r="41">
@@ -2791,7 +2791,7 @@
         </is>
       </c>
       <c r="B41" t="n">
-        <v>-0.04315599143577227</v>
+        <v>-0.03102246861014932</v>
       </c>
     </row>
     <row r="42">
@@ -2801,7 +2801,7 @@
         </is>
       </c>
       <c r="B42" t="n">
-        <v>0.04315599143577227</v>
+        <v>0.03102246861014932</v>
       </c>
     </row>
     <row r="43">
@@ -2811,7 +2811,7 @@
         </is>
       </c>
       <c r="B43" t="n">
-        <v>-0.1440758110043622</v>
+        <v>-0.1100708544316998</v>
       </c>
     </row>
     <row r="44">
@@ -2821,7 +2821,7 @@
         </is>
       </c>
       <c r="B44" t="n">
-        <v>1.152606476527654</v>
+        <v>0.8805668266490886</v>
       </c>
     </row>
     <row r="45">
@@ -2831,7 +2831,7 @@
         </is>
       </c>
       <c r="B45" t="n">
-        <v>-2.179413077165105e-18</v>
+        <v>-3.846850640809567e-18</v>
       </c>
     </row>
     <row r="46">
@@ -2841,7 +2841,7 @@
         </is>
       </c>
       <c r="B46" t="n">
-        <v>2.179413077165105e-18</v>
+        <v>3.846850640809567e-18</v>
       </c>
     </row>
     <row r="47">
@@ -2851,7 +2851,7 @@
         </is>
       </c>
       <c r="B47" t="n">
-        <v>-1.15334136985157e-18</v>
+        <v>-1.15270597288779e-18</v>
       </c>
     </row>
     <row r="48">
@@ -2861,7 +2861,7 @@
         </is>
       </c>
       <c r="B48" t="n">
-        <v>-3.567222967248125e-17</v>
+        <v>-8.494544710917492e-17</v>
       </c>
     </row>
     <row r="49">
@@ -2873,11 +2873,11 @@
       <c r="B49" t="inlineStr">
         <is>
           <t>[AeroComponentResults(
-	L=0.000314036243216673,
+	L=0.000352616649762903,
 	Y=0.0,
-	D=0.0007289501622465802,
+	D=0.0007855778511405799,
 	l_b=0.0,
-	m_b=-2.9076860385309108e-05,
+	m_b=-3.539309727233035e-05,
 	n_b=-0.0,
 	span_effective=0.004055451774444796, oswalds_efficiency=0.95,
 )]</t>
@@ -2891,7 +2891,7 @@
         </is>
       </c>
       <c r="B50" t="n">
-        <v>-2.179413077165105e-18</v>
+        <v>-3.846850640809567e-18</v>
       </c>
     </row>
     <row r="51">
@@ -2901,7 +2901,7 @@
         </is>
       </c>
       <c r="B51" t="n">
-        <v>2.362080122426599e-15</v>
+        <v>1.801817294541999e-14</v>
       </c>
     </row>
     <row r="52">
@@ -2911,7 +2911,7 @@
         </is>
       </c>
       <c r="B52" t="n">
-        <v>1.168760484624072e-17</v>
+        <v>3.00074080998565e-17</v>
       </c>
     </row>
     <row r="53">
@@ -2923,29 +2923,29 @@
       <c r="B53" t="inlineStr">
         <is>
           <t>[AeroComponentResults(
-	L=0.8780379151087044,
+	L=0.7045648921134826,
 	Y=0.0,
-	D=0.06442041737847674,
+	D=0.05434495647015744,
 	l_b=-0.0,
-	m_b=0.08900825386796501,
+	m_b=0.0636749406098028,
 	n_b=-0.0,
-	span_effective=0.9115567574672864, oswalds_efficiency=0.8095875167779147,
+	span_effective=0.7824123147017349, oswalds_efficiency=0.8077792477821385,
 ), AeroComponentResults(
-	L=0.2742545251757332,
+	L=0.17564931788584298,
 	Y=0.0,
-	D=0.02567952455426785,
+	D=0.016244862020259498,
 	l_b=-0.0,
-	m_b=-0.08906211845275344,
+	m_b=-0.06366404685753295,
 	n_b=-0.0,
-	span_effective=0.41637497835985343, oswalds_efficiency=0.8137951483430786,
+	span_effective=0.321907992627013, oswalds_efficiency=0.8106853777008906,
 ), AeroComponentResults(
-	L=-0.0,
-	Y=-3.567222967248125e-17,
-	D=0.0025653343919069247,
-	l_b=-2.1794130771651045e-18,
-	m_b=8.29414451760979e-05,
-	n_b=1.1687604846240722e-17,
-	span_effective=0.15756892889595991, oswalds_efficiency=0.8232692748986458,
+	L=2.710505431213761e-20,
+	Y=-8.494544710917492e-17,
+	D=0.0018054108034454568,
+	l_b=-3.846850640809567e-18,
+	m_b=2.4499345020493072e-05,
+	n_b=3.00074080998565e-17,
+	span_effective=0.11788443735251077, oswalds_efficiency=0.8232692748986458,
 )]</t>
         </is>
       </c>
@@ -2957,7 +2957,7 @@
         </is>
       </c>
       <c r="B54" t="n">
-        <v>0.1578120048746437</v>
+        <v>0.1360978123055108</v>
       </c>
     </row>
     <row r="55">
@@ -2967,7 +2967,7 @@
         </is>
       </c>
       <c r="B55" t="n">
-        <v>0.3081737632218351</v>
+        <v>0.3055745085297195</v>
       </c>
     </row>
     <row r="56">
@@ -2977,7 +2977,7 @@
         </is>
       </c>
       <c r="B56" t="n">
-        <v>0.1418633642512787</v>
+        <v>0.1393928527511432</v>
       </c>
     </row>
     <row r="57">
@@ -2987,7 +2987,7 @@
         </is>
       </c>
       <c r="B57" t="n">
-        <v>0.7071245061333374</v>
+        <v>0.6677777267646771</v>
       </c>
     </row>
     <row r="58">
@@ -2997,7 +2997,7 @@
         </is>
       </c>
       <c r="B58" t="n">
-        <v>2.990596526940585e-17</v>
+        <v>5.789581195068685e-18</v>
       </c>
     </row>
     <row r="59">
@@ -3007,7 +3007,7 @@
         </is>
       </c>
       <c r="B59" t="n">
-        <v>1.931869213079225e-18</v>
+        <v>3.734649104488625e-19</v>
       </c>
     </row>
     <row r="60">
@@ -3017,7 +3017,7 @@
         </is>
       </c>
       <c r="B60" t="n">
-        <v>5.914511041849252e-15</v>
+        <v>-2.261620206498122e-11</v>
       </c>
     </row>
     <row r="61">
@@ -3027,7 +3027,7 @@
         </is>
       </c>
       <c r="B61" t="n">
-        <v>-1.010300013270307e-17</v>
+        <v>-2.899578372353855e-18</v>
       </c>
     </row>
     <row r="62">
@@ -3037,7 +3037,7 @@
         </is>
       </c>
       <c r="B62" t="n">
-        <v>0.2949844355523568</v>
+        <v>0.2093797551446262</v>
       </c>
     </row>
     <row r="63">
@@ -3047,7 +3047,7 @@
         </is>
       </c>
       <c r="B63" t="n">
-        <v>0.09935617363132208</v>
+        <v>0.05994237243079437</v>
       </c>
     </row>
     <row r="64">
@@ -3057,7 +3057,7 @@
         </is>
       </c>
       <c r="B64" t="n">
-        <v>0.1956282619210346</v>
+        <v>0.1494373827138319</v>
       </c>
     </row>
     <row r="65">
@@ -3067,7 +3067,7 @@
         </is>
       </c>
       <c r="B65" t="n">
-        <v>-0.08747860705441396</v>
+        <v>-0.07473112296409837</v>
       </c>
     </row>
     <row r="66">
@@ -3077,7 +3077,7 @@
         </is>
       </c>
       <c r="B66" t="n">
-        <v>0.08747860705441396</v>
+        <v>0.07473112296409837</v>
       </c>
     </row>
     <row r="67">
@@ -3087,7 +3087,7 @@
         </is>
       </c>
       <c r="B67" t="n">
-        <v>-0.2949844355523568</v>
+        <v>-0.2093797551446262</v>
       </c>
     </row>
     <row r="68">
@@ -3097,7 +3097,7 @@
         </is>
       </c>
       <c r="B68" t="n">
-        <v>1.470363574188967</v>
+        <v>1.003058149406276</v>
       </c>
     </row>
     <row r="69">
@@ -3107,7 +3107,7 @@
         </is>
       </c>
       <c r="B69" t="n">
-        <v>3.717816371450392e-18</v>
+        <v>4.456329697044344e-19</v>
       </c>
     </row>
     <row r="70">
@@ -3117,7 +3117,7 @@
         </is>
       </c>
       <c r="B70" t="n">
-        <v>-3.717816371450392e-18</v>
+        <v>-4.456329697044344e-19</v>
       </c>
     </row>
     <row r="71">
@@ -3127,7 +3127,7 @@
         </is>
       </c>
       <c r="B71" t="n">
-        <v>9.757090527598963e-19</v>
+        <v>-1.638120095141176e-20</v>
       </c>
     </row>
     <row r="72">
@@ -3137,7 +3137,7 @@
         </is>
       </c>
       <c r="B72" t="n">
-        <v>6.218514787946424e-17</v>
+        <v>8.696436503653317e-18</v>
       </c>
     </row>
     <row r="73">
@@ -3149,11 +3149,11 @@
       <c r="B73" t="inlineStr">
         <is>
           <t>[AeroComponentResults(
-	L=0.0006015902157105119,
+	L=0.0005721440772656707,
 	Y=0.0,
-	D=0.0006763829236288282,
+	D=0.000691597035098835,
 	l_b=0.0,
-	m_b=-4.457904735356192e-05,
+	m_b=-5.134608615884502e-05,
 	n_b=-0.0,
 	span_effective=0.004055451774444796, oswalds_efficiency=0.95,
 )]</t>
@@ -3167,7 +3167,7 @@
         </is>
       </c>
       <c r="B74" t="n">
-        <v>3.717816371450392e-18</v>
+        <v>4.456329697044344e-19</v>
       </c>
     </row>
     <row r="75">
@@ -3177,7 +3177,7 @@
         </is>
       </c>
       <c r="B75" t="n">
-        <v>2.683623993599699e-15</v>
+        <v>-5.945252909498721e-12</v>
       </c>
     </row>
     <row r="76">
@@ -3187,7 +3187,7 @@
         </is>
       </c>
       <c r="B76" t="n">
-        <v>-1.94428789691513e-17</v>
+        <v>-3.459890567522886e-18</v>
       </c>
     </row>
     <row r="77">
@@ -3199,29 +3199,29 @@
       <c r="B77" t="inlineStr">
         <is>
           <t>[AeroComponentResults(
-	L=1.1470933682913842,
+	L=0.819339492848226,
 	Y=0.0,
-	D=0.13452808441524672,
+	D=0.09613428532860471,
 	l_b=-0.0,
-	m_b=0.10912158150324003,
+	m_b=0.06966064861102046,
 	n_b=-0.0,
-	span_effective=0.9115567574672864, oswalds_efficiency=0.8095875167779147,
+	span_effective=0.7824123147017349, oswalds_efficiency=0.8077792477821385,
 ), AeroComponentResults(
-	L=0.3226686156818727,
+	L=0.18314651248078412,
 	Y=0.0,
-	D=0.05817686423775249,
+	D=0.051073690743135086,
 	l_b=-0.0,
-	m_b=-0.10911225766315945,
+	m_b=-0.06960640580774259,
 	n_b=-0.0,
-	span_effective=0.41637497835985343, oswalds_efficiency=0.8137951483430786,
+	span_effective=0.321907992627013, oswalds_efficiency=0.8106853777008906,
 ), AeroComponentResults(
-	L=-5.421010862427522e-20,
-	Y=6.218514787946424e-17,
-	D=0.0022469303444065903,
-	l_b=3.7178163714503916e-18,
-	m_b=3.525520727566548e-05,
-	n_b=-1.9442878969151304e-17,
-	span_effective=0.15756892889595991, oswalds_efficiency=0.8232692748986458,
+	L=-0.0,
+	Y=8.696436503653317e-18,
+	D=0.0015378096069932246,
+	l_b=4.456329697044344e-19,
+	m_b=-2.8967230642786827e-06,
+	n_b=-3.4598905675228862e-18,
+	span_effective=0.11788443735251077, oswalds_efficiency=0.8232692748986458,
 )]</t>
         </is>
       </c>
@@ -3279,10 +3279,10 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>1.152606476527654</v>
+        <v>0.8805668266490886</v>
       </c>
       <c r="C2" t="n">
-        <v>1.050146104056169</v>
+        <v>0.8805668366482111</v>
       </c>
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="n">
@@ -3299,7 +3299,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.1440758110043622</v>
+        <v>0.1100708544316998</v>
       </c>
       <c r="C3" t="n">
         <v>0.001</v>
@@ -3319,7 +3319,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>4.321499743788634e-15</v>
+        <v>5.47347271698509e-14</v>
       </c>
       <c r="C4" t="n">
         <v>0</v>
@@ -3341,7 +3341,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>-9.400956093217906e-19</v>
+        <v>-2.574427574422738e-18</v>
       </c>
       <c r="C5" t="n">
         <v>0</v>
@@ -3363,7 +3363,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>5.041479338892034e-18</v>
+        <v>2.008185553909865e-17</v>
       </c>
       <c r="C6" t="n">
         <v>0</v>
@@ -3385,7 +3385,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.4601451985001849</v>
+        <v>0.4681348832632325</v>
       </c>
       <c r="C7" t="inlineStr"/>
       <c r="D7" t="n">
@@ -3405,7 +3405,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>8.000000079995392</v>
+        <v>7.608325391688213</v>
       </c>
       <c r="C8" t="inlineStr"/>
       <c r="D8" t="n">
@@ -3425,7 +3425,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>0.7071245061333374</v>
+        <v>0.6677777267646771</v>
       </c>
       <c r="C9" t="inlineStr"/>
       <c r="D9" t="n">
@@ -3445,10 +3445,10 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>1.470363574188967</v>
+        <v>1.003058149406276</v>
       </c>
       <c r="C10" t="n">
-        <v>1.470363584188335</v>
+        <v>0.9589431662417057</v>
       </c>
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="n">
@@ -3465,7 +3465,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>5.914511041849252e-15</v>
+        <v>-2.261620206498122e-11</v>
       </c>
       <c r="C11" t="n">
         <v>0</v>
@@ -3487,7 +3487,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>2.393570521135981</v>
+        <v>2.400000023994921</v>
       </c>
       <c r="C12" t="inlineStr"/>
       <c r="D12" t="n">
@@ -3507,7 +3507,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>3.704393795995896</v>
+        <v>4.270061168506224</v>
       </c>
       <c r="C13" t="n">
         <v>0.5817764173314431</v>
@@ -3523,11 +3523,11 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>H-tail tip deflection (diag)</t>
+          <t>H-tail tip deflection proxy (diag)</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>0.8605320307455027</v>
+        <v>0.4929079927997522</v>
       </c>
       <c r="C14" t="inlineStr"/>
       <c r="D14" t="inlineStr"/>
@@ -3541,11 +3541,11 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>H-tail tip deflection allow (diag)</t>
+          <t>H-tail tip deflection proxy allow (diag)</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>0.01665499913439414</v>
+        <v>0.01287631970508052</v>
       </c>
       <c r="C15" t="inlineStr"/>
       <c r="D15" t="inlineStr"/>
@@ -3559,11 +3559,11 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>H-tail deflection penalty (diag)</t>
+          <t>H-tail deflection proxy penalty (diag)</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>128.3627783308596</v>
+        <v>69.49070752484344</v>
       </c>
       <c r="C16" t="inlineStr"/>
       <c r="D16" t="inlineStr"/>
@@ -3581,7 +3581,7 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>7.999999920130635</v>
+        <v>7.999999920010524</v>
       </c>
       <c r="C17" t="n">
         <v>8</v>
@@ -3601,7 +3601,7 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>5.199892746342704</v>
+        <v>6.333919194811074</v>
       </c>
       <c r="C18" t="n">
         <v>2</v>
@@ -3621,7 +3621,7 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>5.199892746342704</v>
+        <v>6.333919194811074</v>
       </c>
       <c r="C19" t="inlineStr"/>
       <c r="D19" t="n">
@@ -3641,7 +3641,7 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>67223.26919679661</v>
+        <v>56310.25292766299</v>
       </c>
       <c r="C20" t="n">
         <v>20000</v>
@@ -3661,7 +3661,7 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>0.04999998999434588</v>
+        <v>0.04999999007341833</v>
       </c>
       <c r="C21" t="n">
         <v>0.05</v>
@@ -3681,7 +3681,7 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>0.04999998999434588</v>
+        <v>0.04999999007341833</v>
       </c>
       <c r="C22" t="inlineStr"/>
       <c r="D22" t="n">
@@ -3701,7 +3701,7 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>0.4999999900064669</v>
+        <v>0.4999999900054579</v>
       </c>
       <c r="C23" t="n">
         <v>0.5</v>
@@ -3721,7 +3721,7 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>0.4999999900064669</v>
+        <v>0.4999999900054579</v>
       </c>
       <c r="C24" t="inlineStr"/>
       <c r="D24" t="n">
@@ -3741,7 +3741,7 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>0.02999999000058427</v>
+        <v>0.02999999000124711</v>
       </c>
       <c r="C25" t="n">
         <v>0.03</v>
@@ -3761,7 +3761,7 @@
         </is>
       </c>
       <c r="B26" t="n">
-        <v>0.02999999000058427</v>
+        <v>0.02999999000124711</v>
       </c>
       <c r="C26" t="inlineStr"/>
       <c r="D26" t="n">
@@ -3781,7 +3781,7 @@
         </is>
       </c>
       <c r="B27" t="n">
-        <v>-0.1497243077168116</v>
+        <v>-0.1588441682609945</v>
       </c>
       <c r="C27" t="inlineStr"/>
       <c r="D27" t="n">
@@ -3801,7 +3801,7 @@
         </is>
       </c>
       <c r="B28" t="n">
-        <v>0.03505599997496323</v>
+        <v>0.0407860197448539</v>
       </c>
       <c r="C28" t="n">
         <v>0</v>
@@ -3821,7 +3821,7 @@
         </is>
       </c>
       <c r="B29" t="n">
-        <v>-6.231079381770853</v>
+        <v>-9.078162866799115</v>
       </c>
       <c r="C29" t="inlineStr"/>
       <c r="D29" t="n">
@@ -3841,7 +3841,7 @@
         </is>
       </c>
       <c r="B30" t="n">
-        <v>4.065798068775985</v>
+        <v>4.778401783804584</v>
       </c>
       <c r="C30" t="n">
         <v>0.6</v>
@@ -3861,7 +3861,7 @@
         </is>
       </c>
       <c r="B31" t="n">
-        <v>162.8965872304802</v>
+        <v>206.9382837941339</v>
       </c>
       <c r="C31" t="n">
         <v>2</v>
@@ -3881,7 +3881,7 @@
         </is>
       </c>
       <c r="B32" t="n">
-        <v>0.02495938151867688</v>
+        <v>0.02309095106132333</v>
       </c>
       <c r="C32" t="inlineStr"/>
       <c r="D32" t="n">
@@ -3901,7 +3901,7 @@
         </is>
       </c>
       <c r="B33" t="n">
-        <v>2.575737283287555e-05</v>
+        <v>1.551276539285925e-05</v>
       </c>
       <c r="C33" t="inlineStr"/>
       <c r="D33" t="n">
@@ -3921,7 +3921,7 @@
         </is>
       </c>
       <c r="B34" t="n">
-        <v>1.72210662448098e-05</v>
+        <v>6.646427043993081e-06</v>
       </c>
       <c r="C34" t="inlineStr"/>
       <c r="D34" t="n">
@@ -3941,7 +3941,7 @@
         </is>
       </c>
       <c r="B35" t="n">
-        <v>3.890340309234259e-06</v>
+        <v>1.777116740371975e-06</v>
       </c>
       <c r="C35" t="inlineStr"/>
       <c r="D35" t="n">
@@ -3961,7 +3961,7 @@
         </is>
       </c>
       <c r="B36" t="n">
-        <v>2.809137900571732e-18</v>
+        <v>5.377062767205443e-18</v>
       </c>
       <c r="C36" t="inlineStr"/>
       <c r="D36" t="n">
@@ -3981,7 +3981,7 @@
         </is>
       </c>
       <c r="B37" t="n">
-        <v>4.149054262853123</v>
+        <v>8.219893660890538</v>
       </c>
       <c r="C37" t="inlineStr"/>
       <c r="D37" t="n">
@@ -4001,7 +4001,7 @@
         </is>
       </c>
       <c r="B38" t="n">
-        <v>7.814204555748593e-17</v>
+        <v>1.454124360923813e-15</v>
       </c>
       <c r="C38" t="inlineStr"/>
       <c r="D38" t="n">
@@ -4082,7 +4082,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>4.995818923191007</v>
+        <v>5.121658855088541</v>
       </c>
       <c r="C2" t="n">
         <v>-4</v>
@@ -4115,7 +4115,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>2.318821944480995e-16</v>
+        <v>-1.003039419388021e-16</v>
       </c>
       <c r="C3" t="n">
         <v>-30</v>
@@ -4148,7 +4148,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>1.248382770292376</v>
+        <v>1.07084831044651</v>
       </c>
       <c r="C4" t="n">
         <v>-30</v>
@@ -4181,7 +4181,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>3.758299667982743e-15</v>
+        <v>7.417831106112554e-15</v>
       </c>
       <c r="C5" t="n">
         <v>-30</v>
@@ -4214,7 +4214,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>8.000000079995392</v>
+        <v>7.608325391688213</v>
       </c>
       <c r="C6" t="n">
         <v>-4</v>
@@ -4232,17 +4232,13 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>upper</t>
+          <t>none</t>
         </is>
       </c>
       <c r="H6" t="b">
-        <v>1</v>
-      </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>[WARN] alpha_turn_deg hit upper bound (value=8, upper=8, tol=0.012).</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="I6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -4251,7 +4247,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>-2.809137900571732e-18</v>
+        <v>5.377062767205443e-18</v>
       </c>
       <c r="C7" t="n">
         <v>-30</v>
@@ -4284,7 +4280,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>4.149054262853123</v>
+        <v>8.219893660890538</v>
       </c>
       <c r="C8" t="n">
         <v>-30</v>
@@ -4317,7 +4313,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>7.814204555748593e-17</v>
+        <v>1.454124360923813e-15</v>
       </c>
       <c r="C9" t="n">
         <v>-30</v>
@@ -4350,7 +4346,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>0.9114499515298465</v>
+        <v>0.7823206404532017</v>
       </c>
       <c r="C10" t="n">
         <v>0.3</v>
@@ -4383,7 +4379,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.2182096598924276</v>
+        <v>0.1750074259201051</v>
       </c>
       <c r="C11" t="n">
         <v>0.1</v>
@@ -4416,7 +4412,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.6440573443182428</v>
+        <v>0.6399411649061671</v>
       </c>
       <c r="C12" t="n">
         <v>0.35</v>
@@ -4449,7 +4445,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.4163749783598534</v>
+        <v>0.321907992627013</v>
       </c>
       <c r="C13" t="n">
         <v>0.2</v>
@@ -4482,7 +4478,7 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>0.1575689288959599</v>
+        <v>0.1178844373525108</v>
       </c>
       <c r="C14" t="n">
         <v>0.1</v>
@@ -4552,7 +4548,7 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>0.6766792150473272</v>
+        <v>0.739374410448861</v>
       </c>
       <c r="C16" t="n">
         <v>0</v>
@@ -4626,7 +4622,7 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>4.5</v>
+        <v>4.7</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -4646,7 +4642,7 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>4.1</v>
+        <v>4.2</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
@@ -4786,7 +4782,7 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>4.995818923191007</v>
+        <v>5.121658855088541</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
@@ -4806,7 +4802,7 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>2.318821944480995e-16</v>
+        <v>-1.003039419388021e-16</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
@@ -4826,7 +4822,7 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>1.248382770292376</v>
+        <v>1.07084831044651</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
@@ -4846,7 +4842,7 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>3.758299667982743e-15</v>
+        <v>7.417831106112554e-15</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
@@ -4866,7 +4862,7 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>0.617381854787086</v>
+        <v>0.5874999992029738</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
@@ -4886,7 +4882,7 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>0.4601451985001849</v>
+        <v>0.4681348832632325</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
@@ -4906,7 +4902,7 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>8.000000079995392</v>
+        <v>7.608325391688213</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
@@ -4926,7 +4922,7 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>-2.809137900571732e-18</v>
+        <v>5.377062767205443e-18</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
@@ -4946,7 +4942,7 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>4.149054262853123</v>
+        <v>8.219893660890538</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
@@ -4966,7 +4962,7 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>7.814204555748593e-17</v>
+        <v>1.454124360923813e-15</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
@@ -4986,7 +4982,7 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>0.7071245061333374</v>
+        <v>0.6677777267646771</v>
       </c>
       <c r="D20" t="inlineStr">
         <is>
@@ -5006,7 +5002,7 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>1.437845545371058</v>
+        <v>1.50883970376832</v>
       </c>
       <c r="D21" t="inlineStr">
         <is>
@@ -5026,7 +5022,7 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>2.393570521135981</v>
+        <v>2.400000023994921</v>
       </c>
       <c r="D22" t="inlineStr">
         <is>

</xml_diff>